<commit_message>
Templates: drop PM history/warranty/units column, set-or-reason and delivery lists, cleaner layout
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz4sTjvfWvU37rjR8pe
</commit_message>
<xml_diff>
--- a/tracker/templates/TEMPLATE_FilterLog.xlsx
+++ b/tracker/templates/TEMPLATE_FilterLog.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filter Log" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Filter Log'!$7:$7</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -27,16 +29,18 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="16"/>
     </font>
     <font>
-      <i val="1"/>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,11 +49,16 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -57,26 +66,59 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00F8CBAD"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00F2F2F2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -440,158 +482,1171 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H14"/>
+  <dimension ref="A1:H107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="26" customWidth="1" min="7" max="7"/>
-    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="45" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FILTER LOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Job number</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Airco PM</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>Project name</t>
         </is>
       </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Airco APM</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Phase</t>
         </is>
       </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr">
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Airco PM</t>
+          <t>GC</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr">
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Airco APM</t>
+          <t>Job type</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr">
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Ordered by</t>
         </is>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
-        <is>
-          <t>GC</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>Job type</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>PM history</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>Warranty expires</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Yellow = still needs info. Red = unit not replaced. One row per filter size (a unit that takes 2 sizes gets 2 rows). Write sizes W x L x D and say if nominal or exact.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Filter size (W x L x D)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C7" s="4" t="inlineStr">
         <is>
           <t>QTY</t>
         </is>
       </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>Filter set installed</t>
+          <t>Filter set or reason</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
         <is>
           <t>MERV</t>
         </is>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>Installed size if different from spec</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="H7" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
     </row>
-    <row r="14"/>
+    <row r="8">
+      <c r="A8" s="5" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="6" t="n"/>
+      <c r="H8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="6" t="n"/>
+      <c r="H14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="6" t="n"/>
+      <c r="H15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="6" t="n"/>
+      <c r="H16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="6" t="n"/>
+      <c r="H17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="6" t="n"/>
+      <c r="H18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="6" t="n"/>
+      <c r="H19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="6" t="n"/>
+      <c r="H20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="6" t="n"/>
+      <c r="H21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="6" t="n"/>
+      <c r="H22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="6" t="n"/>
+      <c r="H23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="6" t="n"/>
+      <c r="H24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="6" t="n"/>
+      <c r="H25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="6" t="n"/>
+      <c r="H26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="6" t="n"/>
+      <c r="H28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="n"/>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="6" t="n"/>
+      <c r="H29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="n"/>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="6" t="n"/>
+      <c r="H31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n"/>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="6" t="n"/>
+      <c r="H32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="n"/>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="6" t="n"/>
+      <c r="H33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="n"/>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="6" t="n"/>
+      <c r="H34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="n"/>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="n"/>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="6" t="n"/>
+      <c r="H36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="n"/>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="6" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="6" t="n"/>
+      <c r="H37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="n"/>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="n"/>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="6" t="n"/>
+      <c r="H40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="n"/>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="6" t="n"/>
+      <c r="H41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="n"/>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="6" t="n"/>
+      <c r="H42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="n"/>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="6" t="n"/>
+      <c r="H43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="n"/>
+      <c r="B44" s="6" t="n"/>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="6" t="n"/>
+      <c r="H44" s="7" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="n"/>
+      <c r="B45" s="6" t="n"/>
+      <c r="C45" s="6" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="6" t="n"/>
+      <c r="H45" s="7" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="n"/>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="6" t="n"/>
+      <c r="H46" s="7" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="n"/>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="6" t="n"/>
+      <c r="H47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="n"/>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="6" t="n"/>
+      <c r="H48" s="7" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="n"/>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="6" t="n"/>
+      <c r="H49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="n"/>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="6" t="n"/>
+      <c r="H50" s="7" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="n"/>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="6" t="n"/>
+      <c r="H51" s="7" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="n"/>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="6" t="n"/>
+      <c r="H52" s="7" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="n"/>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="6" t="n"/>
+      <c r="H53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="n"/>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="6" t="n"/>
+      <c r="H54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="n"/>
+      <c r="B55" s="6" t="n"/>
+      <c r="C55" s="6" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="6" t="n"/>
+      <c r="H55" s="7" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="n"/>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="6" t="n"/>
+      <c r="H56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="5" t="n"/>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="6" t="n"/>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="6" t="n"/>
+      <c r="F57" s="6" t="n"/>
+      <c r="G57" s="6" t="n"/>
+      <c r="H57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="5" t="n"/>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="6" t="n"/>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="6" t="n"/>
+      <c r="F58" s="6" t="n"/>
+      <c r="G58" s="6" t="n"/>
+      <c r="H58" s="7" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="5" t="n"/>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="6" t="n"/>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="6" t="n"/>
+      <c r="F59" s="6" t="n"/>
+      <c r="G59" s="6" t="n"/>
+      <c r="H59" s="7" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="5" t="n"/>
+      <c r="B60" s="6" t="n"/>
+      <c r="C60" s="6" t="n"/>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="6" t="n"/>
+      <c r="F60" s="6" t="n"/>
+      <c r="G60" s="6" t="n"/>
+      <c r="H60" s="7" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="5" t="n"/>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="6" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="6" t="n"/>
+      <c r="F61" s="6" t="n"/>
+      <c r="G61" s="6" t="n"/>
+      <c r="H61" s="7" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="5" t="n"/>
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="6" t="n"/>
+      <c r="E62" s="6" t="n"/>
+      <c r="F62" s="6" t="n"/>
+      <c r="G62" s="6" t="n"/>
+      <c r="H62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="5" t="n"/>
+      <c r="B63" s="6" t="n"/>
+      <c r="C63" s="6" t="n"/>
+      <c r="D63" s="6" t="n"/>
+      <c r="E63" s="6" t="n"/>
+      <c r="F63" s="6" t="n"/>
+      <c r="G63" s="6" t="n"/>
+      <c r="H63" s="7" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="5" t="n"/>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="6" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="6" t="n"/>
+      <c r="G64" s="6" t="n"/>
+      <c r="H64" s="7" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="5" t="n"/>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="6" t="n"/>
+      <c r="G65" s="6" t="n"/>
+      <c r="H65" s="7" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="5" t="n"/>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="6" t="n"/>
+      <c r="G66" s="6" t="n"/>
+      <c r="H66" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="5" t="n"/>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="6" t="n"/>
+      <c r="H67" s="7" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="5" t="n"/>
+      <c r="B68" s="6" t="n"/>
+      <c r="C68" s="6" t="n"/>
+      <c r="D68" s="6" t="n"/>
+      <c r="E68" s="6" t="n"/>
+      <c r="F68" s="6" t="n"/>
+      <c r="G68" s="6" t="n"/>
+      <c r="H68" s="7" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="5" t="n"/>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="6" t="n"/>
+      <c r="D69" s="6" t="n"/>
+      <c r="E69" s="6" t="n"/>
+      <c r="F69" s="6" t="n"/>
+      <c r="G69" s="6" t="n"/>
+      <c r="H69" s="7" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="5" t="n"/>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="6" t="n"/>
+      <c r="D70" s="6" t="n"/>
+      <c r="E70" s="6" t="n"/>
+      <c r="F70" s="6" t="n"/>
+      <c r="G70" s="6" t="n"/>
+      <c r="H70" s="7" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="5" t="n"/>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+      <c r="E71" s="6" t="n"/>
+      <c r="F71" s="6" t="n"/>
+      <c r="G71" s="6" t="n"/>
+      <c r="H71" s="7" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="5" t="n"/>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="6" t="n"/>
+      <c r="D72" s="6" t="n"/>
+      <c r="E72" s="6" t="n"/>
+      <c r="F72" s="6" t="n"/>
+      <c r="G72" s="6" t="n"/>
+      <c r="H72" s="7" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="5" t="n"/>
+      <c r="B73" s="6" t="n"/>
+      <c r="C73" s="6" t="n"/>
+      <c r="D73" s="6" t="n"/>
+      <c r="E73" s="6" t="n"/>
+      <c r="F73" s="6" t="n"/>
+      <c r="G73" s="6" t="n"/>
+      <c r="H73" s="7" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="n"/>
+      <c r="B74" s="6" t="n"/>
+      <c r="C74" s="6" t="n"/>
+      <c r="D74" s="6" t="n"/>
+      <c r="E74" s="6" t="n"/>
+      <c r="F74" s="6" t="n"/>
+      <c r="G74" s="6" t="n"/>
+      <c r="H74" s="7" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="n"/>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="6" t="n"/>
+      <c r="F75" s="6" t="n"/>
+      <c r="G75" s="6" t="n"/>
+      <c r="H75" s="7" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="n"/>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
+      <c r="F76" s="6" t="n"/>
+      <c r="G76" s="6" t="n"/>
+      <c r="H76" s="7" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="5" t="n"/>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="7" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="5" t="n"/>
+      <c r="B78" s="6" t="n"/>
+      <c r="C78" s="6" t="n"/>
+      <c r="D78" s="6" t="n"/>
+      <c r="E78" s="6" t="n"/>
+      <c r="F78" s="6" t="n"/>
+      <c r="G78" s="6" t="n"/>
+      <c r="H78" s="7" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="5" t="n"/>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="6" t="n"/>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="6" t="n"/>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="7" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="5" t="n"/>
+      <c r="B80" s="6" t="n"/>
+      <c r="C80" s="6" t="n"/>
+      <c r="D80" s="6" t="n"/>
+      <c r="E80" s="6" t="n"/>
+      <c r="F80" s="6" t="n"/>
+      <c r="G80" s="6" t="n"/>
+      <c r="H80" s="7" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="5" t="n"/>
+      <c r="B81" s="6" t="n"/>
+      <c r="C81" s="6" t="n"/>
+      <c r="D81" s="6" t="n"/>
+      <c r="E81" s="6" t="n"/>
+      <c r="F81" s="6" t="n"/>
+      <c r="G81" s="6" t="n"/>
+      <c r="H81" s="7" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="5" t="n"/>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="6" t="n"/>
+      <c r="D82" s="6" t="n"/>
+      <c r="E82" s="6" t="n"/>
+      <c r="F82" s="6" t="n"/>
+      <c r="G82" s="6" t="n"/>
+      <c r="H82" s="7" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="5" t="n"/>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
+      <c r="E83" s="6" t="n"/>
+      <c r="F83" s="6" t="n"/>
+      <c r="G83" s="6" t="n"/>
+      <c r="H83" s="7" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="5" t="n"/>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="6" t="n"/>
+      <c r="D84" s="6" t="n"/>
+      <c r="E84" s="6" t="n"/>
+      <c r="F84" s="6" t="n"/>
+      <c r="G84" s="6" t="n"/>
+      <c r="H84" s="7" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="5" t="n"/>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="6" t="n"/>
+      <c r="E85" s="6" t="n"/>
+      <c r="F85" s="6" t="n"/>
+      <c r="G85" s="6" t="n"/>
+      <c r="H85" s="7" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="5" t="n"/>
+      <c r="B86" s="6" t="n"/>
+      <c r="C86" s="6" t="n"/>
+      <c r="D86" s="6" t="n"/>
+      <c r="E86" s="6" t="n"/>
+      <c r="F86" s="6" t="n"/>
+      <c r="G86" s="6" t="n"/>
+      <c r="H86" s="7" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="5" t="n"/>
+      <c r="B87" s="6" t="n"/>
+      <c r="C87" s="6" t="n"/>
+      <c r="D87" s="6" t="n"/>
+      <c r="E87" s="6" t="n"/>
+      <c r="F87" s="6" t="n"/>
+      <c r="G87" s="6" t="n"/>
+      <c r="H87" s="7" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="5" t="n"/>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="6" t="n"/>
+      <c r="D88" s="6" t="n"/>
+      <c r="E88" s="6" t="n"/>
+      <c r="F88" s="6" t="n"/>
+      <c r="G88" s="6" t="n"/>
+      <c r="H88" s="7" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="5" t="n"/>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="6" t="n"/>
+      <c r="F89" s="6" t="n"/>
+      <c r="G89" s="6" t="n"/>
+      <c r="H89" s="7" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="5" t="n"/>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="6" t="n"/>
+      <c r="D90" s="6" t="n"/>
+      <c r="E90" s="6" t="n"/>
+      <c r="F90" s="6" t="n"/>
+      <c r="G90" s="6" t="n"/>
+      <c r="H90" s="7" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="5" t="n"/>
+      <c r="B91" s="6" t="n"/>
+      <c r="C91" s="6" t="n"/>
+      <c r="D91" s="6" t="n"/>
+      <c r="E91" s="6" t="n"/>
+      <c r="F91" s="6" t="n"/>
+      <c r="G91" s="6" t="n"/>
+      <c r="H91" s="7" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="5" t="n"/>
+      <c r="B92" s="6" t="n"/>
+      <c r="C92" s="6" t="n"/>
+      <c r="D92" s="6" t="n"/>
+      <c r="E92" s="6" t="n"/>
+      <c r="F92" s="6" t="n"/>
+      <c r="G92" s="6" t="n"/>
+      <c r="H92" s="7" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="5" t="n"/>
+      <c r="B93" s="6" t="n"/>
+      <c r="C93" s="6" t="n"/>
+      <c r="D93" s="6" t="n"/>
+      <c r="E93" s="6" t="n"/>
+      <c r="F93" s="6" t="n"/>
+      <c r="G93" s="6" t="n"/>
+      <c r="H93" s="7" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="5" t="n"/>
+      <c r="B94" s="6" t="n"/>
+      <c r="C94" s="6" t="n"/>
+      <c r="D94" s="6" t="n"/>
+      <c r="E94" s="6" t="n"/>
+      <c r="F94" s="6" t="n"/>
+      <c r="G94" s="6" t="n"/>
+      <c r="H94" s="7" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="5" t="n"/>
+      <c r="B95" s="6" t="n"/>
+      <c r="C95" s="6" t="n"/>
+      <c r="D95" s="6" t="n"/>
+      <c r="E95" s="6" t="n"/>
+      <c r="F95" s="6" t="n"/>
+      <c r="G95" s="6" t="n"/>
+      <c r="H95" s="7" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="5" t="n"/>
+      <c r="B96" s="6" t="n"/>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="6" t="n"/>
+      <c r="F96" s="6" t="n"/>
+      <c r="G96" s="6" t="n"/>
+      <c r="H96" s="7" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="5" t="n"/>
+      <c r="B97" s="6" t="n"/>
+      <c r="C97" s="6" t="n"/>
+      <c r="D97" s="6" t="n"/>
+      <c r="E97" s="6" t="n"/>
+      <c r="F97" s="6" t="n"/>
+      <c r="G97" s="6" t="n"/>
+      <c r="H97" s="7" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="5" t="n"/>
+      <c r="B98" s="6" t="n"/>
+      <c r="C98" s="6" t="n"/>
+      <c r="D98" s="6" t="n"/>
+      <c r="E98" s="6" t="n"/>
+      <c r="F98" s="6" t="n"/>
+      <c r="G98" s="6" t="n"/>
+      <c r="H98" s="7" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="5" t="n"/>
+      <c r="B99" s="6" t="n"/>
+      <c r="C99" s="6" t="n"/>
+      <c r="D99" s="6" t="n"/>
+      <c r="E99" s="6" t="n"/>
+      <c r="F99" s="6" t="n"/>
+      <c r="G99" s="6" t="n"/>
+      <c r="H99" s="7" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="5" t="n"/>
+      <c r="B100" s="6" t="n"/>
+      <c r="C100" s="6" t="n"/>
+      <c r="D100" s="6" t="n"/>
+      <c r="E100" s="6" t="n"/>
+      <c r="F100" s="6" t="n"/>
+      <c r="G100" s="6" t="n"/>
+      <c r="H100" s="7" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="5" t="n"/>
+      <c r="B101" s="6" t="n"/>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="6" t="n"/>
+      <c r="F101" s="6" t="n"/>
+      <c r="G101" s="6" t="n"/>
+      <c r="H101" s="7" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="5" t="n"/>
+      <c r="B102" s="6" t="n"/>
+      <c r="C102" s="6" t="n"/>
+      <c r="D102" s="6" t="n"/>
+      <c r="E102" s="6" t="n"/>
+      <c r="F102" s="6" t="n"/>
+      <c r="G102" s="6" t="n"/>
+      <c r="H102" s="7" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="5" t="n"/>
+      <c r="B103" s="6" t="n"/>
+      <c r="C103" s="6" t="n"/>
+      <c r="D103" s="6" t="n"/>
+      <c r="E103" s="6" t="n"/>
+      <c r="F103" s="6" t="n"/>
+      <c r="G103" s="6" t="n"/>
+      <c r="H103" s="7" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="5" t="n"/>
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="n"/>
+      <c r="D104" s="6" t="n"/>
+      <c r="E104" s="6" t="n"/>
+      <c r="F104" s="6" t="n"/>
+      <c r="G104" s="6" t="n"/>
+      <c r="H104" s="7" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="5" t="n"/>
+      <c r="B105" s="6" t="n"/>
+      <c r="C105" s="6" t="n"/>
+      <c r="D105" s="6" t="n"/>
+      <c r="E105" s="6" t="n"/>
+      <c r="F105" s="6" t="n"/>
+      <c r="G105" s="6" t="n"/>
+      <c r="H105" s="7" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="5" t="n"/>
+      <c r="B106" s="6" t="n"/>
+      <c r="C106" s="6" t="n"/>
+      <c r="D106" s="6" t="n"/>
+      <c r="E106" s="6" t="n"/>
+      <c r="F106" s="6" t="n"/>
+      <c r="G106" s="6" t="n"/>
+      <c r="H106" s="7" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="5" t="n"/>
+      <c r="B107" s="6" t="n"/>
+      <c r="C107" s="6" t="n"/>
+      <c r="D107" s="6" t="n"/>
+      <c r="E107" s="6" t="n"/>
+      <c r="F107" s="6" t="n"/>
+      <c r="G107" s="6" t="n"/>
+      <c r="H107" s="7" t="n"/>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D14:D113">
-    <cfRule type="expression" priority="1" dxfId="0">
-      <formula>$D14="Not replaced"</formula>
+  <mergeCells count="9">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="F5:H5"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="F4:H4"/>
+    <mergeCell ref="F2:H2"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="F3:H3"/>
+    <mergeCell ref="B4:C4"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A8:H107">
+    <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
+      <formula>$D8="Not replaced"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
-    <dataValidation sqref="D14:D113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D8:D107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not started,Needs filters,Ordered,Replaced,Not replaced,Washable - not replaced"</formula1>
     </dataValidation>
-    <dataValidation sqref="E14:E113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"1,2,3,Attic"</formula1>
+    <dataValidation sqref="E8:E107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1st (media roll),2nd,3rd,Attic stock,RFI,Change order"</formula1>
     </dataValidation>
-    <dataValidation sqref="F14:F113" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F8:F107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"8,13"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Templates: Filter Log and Filter Orders as two tabs of one file
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz4sTjvfWvU37rjR8pe
</commit_message>
<xml_diff>
--- a/tracker/templates/TEMPLATE_FilterLog.xlsx
+++ b/tracker/templates/TEMPLATE_FilterLog.xlsx
@@ -8,9 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filter Log" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Filter Orders" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Filter Log'!$7:$7</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Filter Orders'!$7:$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -18,7 +20,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
+    <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.00"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -84,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -102,6 +107,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1649,4 +1660,1328 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M67"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>FILTER ORDERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Job number</t>
+        </is>
+      </c>
+      <c r="B2" s="3">
+        <f>IF('Filter Log'!B2="","",'Filter Log'!B2)</f>
+        <v/>
+      </c>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Airco PM</t>
+        </is>
+      </c>
+      <c r="H2" s="3">
+        <f>IF('Filter Log'!F2="","",'Filter Log'!F2)</f>
+        <v/>
+      </c>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="20" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Project name</t>
+        </is>
+      </c>
+      <c r="B3" s="3">
+        <f>IF('Filter Log'!B3="","",'Filter Log'!B3)</f>
+        <v/>
+      </c>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Airco APM</t>
+        </is>
+      </c>
+      <c r="H3" s="3">
+        <f>IF('Filter Log'!F3="","",'Filter Log'!F3)</f>
+        <v/>
+      </c>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="B4" s="3">
+        <f>IF('Filter Log'!B4="","",'Filter Log'!B4)</f>
+        <v/>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="H4" s="3">
+        <f>IF('Filter Log'!F4="","",'Filter Log'!F4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
+      <c r="M4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Job type</t>
+        </is>
+      </c>
+      <c r="B5" s="3">
+        <f>IF('Filter Log'!B5="","",'Filter Log'!B5)</f>
+        <v/>
+      </c>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Ordered by</t>
+        </is>
+      </c>
+      <c r="H5" s="3">
+        <f>IF('Filter Log'!F5="","",'Filter Log'!F5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="8" customHeight="1"/>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Order date</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Filter set or reason</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Vendor</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Vendor SO #</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Our PO #</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>MERV</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>Order total price</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>Size</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>QTY</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Unit price</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Line total</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Delivery</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="7" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+      <c r="F8" s="6" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="6" t="n"/>
+      <c r="I8" s="6" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="9">
+        <f>IF(OR(I8="",J8=""),"",I8*J8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="7" t="n"/>
+      <c r="M8" s="7" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="7" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="9" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="9">
+        <f>IF(OR(I9="",J9=""),"",I9*J9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="7" t="n"/>
+      <c r="M9" s="7" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="7" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="9" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="9">
+        <f>IF(OR(I10="",J10=""),"",I10*J10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="7" t="n"/>
+      <c r="M10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="7" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="9" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="9">
+        <f>IF(OR(I11="",J11=""),"",I11*J11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="7" t="n"/>
+      <c r="M11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9">
+        <f>IF(OR(I12="",J12=""),"",I12*J12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="7" t="n"/>
+      <c r="M12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="7" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="9" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="9">
+        <f>IF(OR(I13="",J13=""),"",I13*J13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="7" t="n"/>
+      <c r="M13" s="7" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="7" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+      <c r="F14" s="6" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="6" t="n"/>
+      <c r="I14" s="6" t="n"/>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="9">
+        <f>IF(OR(I14="",J14=""),"",I14*J14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="7" t="n"/>
+      <c r="M14" s="7" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="7" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+      <c r="F15" s="6" t="n"/>
+      <c r="G15" s="9" t="n"/>
+      <c r="H15" s="6" t="n"/>
+      <c r="I15" s="6" t="n"/>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="9">
+        <f>IF(OR(I15="",J15=""),"",I15*J15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="7" t="n"/>
+      <c r="M15" s="7" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+      <c r="F16" s="6" t="n"/>
+      <c r="G16" s="9" t="n"/>
+      <c r="H16" s="6" t="n"/>
+      <c r="I16" s="6" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="9">
+        <f>IF(OR(I16="",J16=""),"",I16*J16)</f>
+        <v/>
+      </c>
+      <c r="L16" s="7" t="n"/>
+      <c r="M16" s="7" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="7" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+      <c r="F17" s="6" t="n"/>
+      <c r="G17" s="9" t="n"/>
+      <c r="H17" s="6" t="n"/>
+      <c r="I17" s="6" t="n"/>
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="9">
+        <f>IF(OR(I17="",J17=""),"",I17*J17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="7" t="n"/>
+      <c r="M17" s="7" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="7" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+      <c r="F18" s="6" t="n"/>
+      <c r="G18" s="9" t="n"/>
+      <c r="H18" s="6" t="n"/>
+      <c r="I18" s="6" t="n"/>
+      <c r="J18" s="9" t="n"/>
+      <c r="K18" s="9">
+        <f>IF(OR(I18="",J18=""),"",I18*J18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="7" t="n"/>
+      <c r="M18" s="7" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="7" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+      <c r="F19" s="6" t="n"/>
+      <c r="G19" s="9" t="n"/>
+      <c r="H19" s="6" t="n"/>
+      <c r="I19" s="6" t="n"/>
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="9">
+        <f>IF(OR(I19="",J19=""),"",I19*J19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="7" t="n"/>
+      <c r="M19" s="7" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="7" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+      <c r="F20" s="6" t="n"/>
+      <c r="G20" s="9" t="n"/>
+      <c r="H20" s="6" t="n"/>
+      <c r="I20" s="6" t="n"/>
+      <c r="J20" s="9" t="n"/>
+      <c r="K20" s="9">
+        <f>IF(OR(I20="",J20=""),"",I20*J20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="7" t="n"/>
+      <c r="M20" s="7" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="7" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+      <c r="F21" s="6" t="n"/>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="6" t="n"/>
+      <c r="I21" s="6" t="n"/>
+      <c r="J21" s="9" t="n"/>
+      <c r="K21" s="9">
+        <f>IF(OR(I21="",J21=""),"",I21*J21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="7" t="n"/>
+      <c r="M21" s="7" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="7" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+      <c r="F22" s="6" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="6" t="n"/>
+      <c r="I22" s="6" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9">
+        <f>IF(OR(I22="",J22=""),"",I22*J22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="7" t="n"/>
+      <c r="M22" s="7" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="7" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+      <c r="F23" s="6" t="n"/>
+      <c r="G23" s="9" t="n"/>
+      <c r="H23" s="6" t="n"/>
+      <c r="I23" s="6" t="n"/>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="9">
+        <f>IF(OR(I23="",J23=""),"",I23*J23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="7" t="n"/>
+      <c r="M23" s="7" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="7" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+      <c r="F24" s="6" t="n"/>
+      <c r="G24" s="9" t="n"/>
+      <c r="H24" s="6" t="n"/>
+      <c r="I24" s="6" t="n"/>
+      <c r="J24" s="9" t="n"/>
+      <c r="K24" s="9">
+        <f>IF(OR(I24="",J24=""),"",I24*J24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="7" t="n"/>
+      <c r="M24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="7" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+      <c r="F25" s="6" t="n"/>
+      <c r="G25" s="9" t="n"/>
+      <c r="H25" s="6" t="n"/>
+      <c r="I25" s="6" t="n"/>
+      <c r="J25" s="9" t="n"/>
+      <c r="K25" s="9">
+        <f>IF(OR(I25="",J25=""),"",I25*J25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="7" t="n"/>
+      <c r="M25" s="7" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="7" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+      <c r="F26" s="6" t="n"/>
+      <c r="G26" s="9" t="n"/>
+      <c r="H26" s="6" t="n"/>
+      <c r="I26" s="6" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="9">
+        <f>IF(OR(I26="",J26=""),"",I26*J26)</f>
+        <v/>
+      </c>
+      <c r="L26" s="7" t="n"/>
+      <c r="M26" s="7" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="7" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="9" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="9" t="n"/>
+      <c r="K27" s="9">
+        <f>IF(OR(I27="",J27=""),"",I27*J27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="7" t="n"/>
+      <c r="M27" s="7" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="7" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
+      <c r="F28" s="6" t="n"/>
+      <c r="G28" s="9" t="n"/>
+      <c r="H28" s="6" t="n"/>
+      <c r="I28" s="6" t="n"/>
+      <c r="J28" s="9" t="n"/>
+      <c r="K28" s="9">
+        <f>IF(OR(I28="",J28=""),"",I28*J28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="7" t="n"/>
+      <c r="M28" s="7" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="7" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+      <c r="F29" s="6" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="6" t="n"/>
+      <c r="I29" s="6" t="n"/>
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="9">
+        <f>IF(OR(I29="",J29=""),"",I29*J29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="7" t="n"/>
+      <c r="M29" s="7" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="7" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n"/>
+      <c r="F30" s="6" t="n"/>
+      <c r="G30" s="9" t="n"/>
+      <c r="H30" s="6" t="n"/>
+      <c r="I30" s="6" t="n"/>
+      <c r="J30" s="9" t="n"/>
+      <c r="K30" s="9">
+        <f>IF(OR(I30="",J30=""),"",I30*J30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="7" t="n"/>
+      <c r="M30" s="7" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+      <c r="F31" s="6" t="n"/>
+      <c r="G31" s="9" t="n"/>
+      <c r="H31" s="6" t="n"/>
+      <c r="I31" s="6" t="n"/>
+      <c r="J31" s="9" t="n"/>
+      <c r="K31" s="9">
+        <f>IF(OR(I31="",J31=""),"",I31*J31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="7" t="n"/>
+      <c r="M31" s="7" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="6" t="n"/>
+      <c r="F32" s="6" t="n"/>
+      <c r="G32" s="9" t="n"/>
+      <c r="H32" s="6" t="n"/>
+      <c r="I32" s="6" t="n"/>
+      <c r="J32" s="9" t="n"/>
+      <c r="K32" s="9">
+        <f>IF(OR(I32="",J32=""),"",I32*J32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="7" t="n"/>
+      <c r="M32" s="7" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="7" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="6" t="n"/>
+      <c r="F33" s="6" t="n"/>
+      <c r="G33" s="9" t="n"/>
+      <c r="H33" s="6" t="n"/>
+      <c r="I33" s="6" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="9">
+        <f>IF(OR(I33="",J33=""),"",I33*J33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="7" t="n"/>
+      <c r="M33" s="7" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="7" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="6" t="n"/>
+      <c r="F34" s="6" t="n"/>
+      <c r="G34" s="9" t="n"/>
+      <c r="H34" s="6" t="n"/>
+      <c r="I34" s="6" t="n"/>
+      <c r="J34" s="9" t="n"/>
+      <c r="K34" s="9">
+        <f>IF(OR(I34="",J34=""),"",I34*J34)</f>
+        <v/>
+      </c>
+      <c r="L34" s="7" t="n"/>
+      <c r="M34" s="7" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="7" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="9" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="9">
+        <f>IF(OR(I35="",J35=""),"",I35*J35)</f>
+        <v/>
+      </c>
+      <c r="L35" s="7" t="n"/>
+      <c r="M35" s="7" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="7" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
+      <c r="F36" s="6" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="6" t="n"/>
+      <c r="I36" s="6" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="9">
+        <f>IF(OR(I36="",J36=""),"",I36*J36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="7" t="n"/>
+      <c r="M36" s="7" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="7" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="6" t="n"/>
+      <c r="F37" s="6" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="6" t="n"/>
+      <c r="I37" s="6" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="9">
+        <f>IF(OR(I37="",J37=""),"",I37*J37)</f>
+        <v/>
+      </c>
+      <c r="L37" s="7" t="n"/>
+      <c r="M37" s="7" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="7" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="6" t="n"/>
+      <c r="F38" s="6" t="n"/>
+      <c r="G38" s="9" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="n"/>
+      <c r="J38" s="9" t="n"/>
+      <c r="K38" s="9">
+        <f>IF(OR(I38="",J38=""),"",I38*J38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="7" t="n"/>
+      <c r="M38" s="7" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="7" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
+      <c r="F39" s="6" t="n"/>
+      <c r="G39" s="9" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="9">
+        <f>IF(OR(I39="",J39=""),"",I39*J39)</f>
+        <v/>
+      </c>
+      <c r="L39" s="7" t="n"/>
+      <c r="M39" s="7" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+      <c r="F40" s="6" t="n"/>
+      <c r="G40" s="9" t="n"/>
+      <c r="H40" s="6" t="n"/>
+      <c r="I40" s="6" t="n"/>
+      <c r="J40" s="9" t="n"/>
+      <c r="K40" s="9">
+        <f>IF(OR(I40="",J40=""),"",I40*J40)</f>
+        <v/>
+      </c>
+      <c r="L40" s="7" t="n"/>
+      <c r="M40" s="7" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="7" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+      <c r="F41" s="6" t="n"/>
+      <c r="G41" s="9" t="n"/>
+      <c r="H41" s="6" t="n"/>
+      <c r="I41" s="6" t="n"/>
+      <c r="J41" s="9" t="n"/>
+      <c r="K41" s="9">
+        <f>IF(OR(I41="",J41=""),"",I41*J41)</f>
+        <v/>
+      </c>
+      <c r="L41" s="7" t="n"/>
+      <c r="M41" s="7" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="7" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
+      <c r="F42" s="6" t="n"/>
+      <c r="G42" s="9" t="n"/>
+      <c r="H42" s="6" t="n"/>
+      <c r="I42" s="6" t="n"/>
+      <c r="J42" s="9" t="n"/>
+      <c r="K42" s="9">
+        <f>IF(OR(I42="",J42=""),"",I42*J42)</f>
+        <v/>
+      </c>
+      <c r="L42" s="7" t="n"/>
+      <c r="M42" s="7" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="7" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+      <c r="F43" s="6" t="n"/>
+      <c r="G43" s="9" t="n"/>
+      <c r="H43" s="6" t="n"/>
+      <c r="I43" s="6" t="n"/>
+      <c r="J43" s="9" t="n"/>
+      <c r="K43" s="9">
+        <f>IF(OR(I43="",J43=""),"",I43*J43)</f>
+        <v/>
+      </c>
+      <c r="L43" s="7" t="n"/>
+      <c r="M43" s="7" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="6" t="n"/>
+      <c r="C44" s="7" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
+      <c r="F44" s="6" t="n"/>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="6" t="n"/>
+      <c r="I44" s="6" t="n"/>
+      <c r="J44" s="9" t="n"/>
+      <c r="K44" s="9">
+        <f>IF(OR(I44="",J44=""),"",I44*J44)</f>
+        <v/>
+      </c>
+      <c r="L44" s="7" t="n"/>
+      <c r="M44" s="7" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="6" t="n"/>
+      <c r="C45" s="7" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="n"/>
+      <c r="F45" s="6" t="n"/>
+      <c r="G45" s="9" t="n"/>
+      <c r="H45" s="6" t="n"/>
+      <c r="I45" s="6" t="n"/>
+      <c r="J45" s="9" t="n"/>
+      <c r="K45" s="9">
+        <f>IF(OR(I45="",J45=""),"",I45*J45)</f>
+        <v/>
+      </c>
+      <c r="L45" s="7" t="n"/>
+      <c r="M45" s="7" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="7" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+      <c r="F46" s="6" t="n"/>
+      <c r="G46" s="9" t="n"/>
+      <c r="H46" s="6" t="n"/>
+      <c r="I46" s="6" t="n"/>
+      <c r="J46" s="9" t="n"/>
+      <c r="K46" s="9">
+        <f>IF(OR(I46="",J46=""),"",I46*J46)</f>
+        <v/>
+      </c>
+      <c r="L46" s="7" t="n"/>
+      <c r="M46" s="7" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="8" t="n"/>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="7" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+      <c r="F47" s="6" t="n"/>
+      <c r="G47" s="9" t="n"/>
+      <c r="H47" s="6" t="n"/>
+      <c r="I47" s="6" t="n"/>
+      <c r="J47" s="9" t="n"/>
+      <c r="K47" s="9">
+        <f>IF(OR(I47="",J47=""),"",I47*J47)</f>
+        <v/>
+      </c>
+      <c r="L47" s="7" t="n"/>
+      <c r="M47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+      <c r="F48" s="6" t="n"/>
+      <c r="G48" s="9" t="n"/>
+      <c r="H48" s="6" t="n"/>
+      <c r="I48" s="6" t="n"/>
+      <c r="J48" s="9" t="n"/>
+      <c r="K48" s="9">
+        <f>IF(OR(I48="",J48=""),"",I48*J48)</f>
+        <v/>
+      </c>
+      <c r="L48" s="7" t="n"/>
+      <c r="M48" s="7" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="7" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+      <c r="F49" s="6" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="6" t="n"/>
+      <c r="I49" s="6" t="n"/>
+      <c r="J49" s="9" t="n"/>
+      <c r="K49" s="9">
+        <f>IF(OR(I49="",J49=""),"",I49*J49)</f>
+        <v/>
+      </c>
+      <c r="L49" s="7" t="n"/>
+      <c r="M49" s="7" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="n"/>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="7" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n"/>
+      <c r="G50" s="9" t="n"/>
+      <c r="H50" s="6" t="n"/>
+      <c r="I50" s="6" t="n"/>
+      <c r="J50" s="9" t="n"/>
+      <c r="K50" s="9">
+        <f>IF(OR(I50="",J50=""),"",I50*J50)</f>
+        <v/>
+      </c>
+      <c r="L50" s="7" t="n"/>
+      <c r="M50" s="7" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="n"/>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+      <c r="F51" s="6" t="n"/>
+      <c r="G51" s="9" t="n"/>
+      <c r="H51" s="6" t="n"/>
+      <c r="I51" s="6" t="n"/>
+      <c r="J51" s="9" t="n"/>
+      <c r="K51" s="9">
+        <f>IF(OR(I51="",J51=""),"",I51*J51)</f>
+        <v/>
+      </c>
+      <c r="L51" s="7" t="n"/>
+      <c r="M51" s="7" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="8" t="n"/>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="7" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n"/>
+      <c r="G52" s="9" t="n"/>
+      <c r="H52" s="6" t="n"/>
+      <c r="I52" s="6" t="n"/>
+      <c r="J52" s="9" t="n"/>
+      <c r="K52" s="9">
+        <f>IF(OR(I52="",J52=""),"",I52*J52)</f>
+        <v/>
+      </c>
+      <c r="L52" s="7" t="n"/>
+      <c r="M52" s="7" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="n"/>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="7" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+      <c r="F53" s="6" t="n"/>
+      <c r="G53" s="9" t="n"/>
+      <c r="H53" s="6" t="n"/>
+      <c r="I53" s="6" t="n"/>
+      <c r="J53" s="9" t="n"/>
+      <c r="K53" s="9">
+        <f>IF(OR(I53="",J53=""),"",I53*J53)</f>
+        <v/>
+      </c>
+      <c r="L53" s="7" t="n"/>
+      <c r="M53" s="7" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="7" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
+      <c r="F54" s="6" t="n"/>
+      <c r="G54" s="9" t="n"/>
+      <c r="H54" s="6" t="n"/>
+      <c r="I54" s="6" t="n"/>
+      <c r="J54" s="9" t="n"/>
+      <c r="K54" s="9">
+        <f>IF(OR(I54="",J54=""),"",I54*J54)</f>
+        <v/>
+      </c>
+      <c r="L54" s="7" t="n"/>
+      <c r="M54" s="7" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="n"/>
+      <c r="B55" s="6" t="n"/>
+      <c r="C55" s="7" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
+      <c r="F55" s="6" t="n"/>
+      <c r="G55" s="9" t="n"/>
+      <c r="H55" s="6" t="n"/>
+      <c r="I55" s="6" t="n"/>
+      <c r="J55" s="9" t="n"/>
+      <c r="K55" s="9">
+        <f>IF(OR(I55="",J55=""),"",I55*J55)</f>
+        <v/>
+      </c>
+      <c r="L55" s="7" t="n"/>
+      <c r="M55" s="7" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="7" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
+      <c r="F56" s="6" t="n"/>
+      <c r="G56" s="9" t="n"/>
+      <c r="H56" s="6" t="n"/>
+      <c r="I56" s="6" t="n"/>
+      <c r="J56" s="9" t="n"/>
+      <c r="K56" s="9">
+        <f>IF(OR(I56="",J56=""),"",I56*J56)</f>
+        <v/>
+      </c>
+      <c r="L56" s="7" t="n"/>
+      <c r="M56" s="7" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="8" t="n"/>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="7" t="n"/>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="6" t="n"/>
+      <c r="F57" s="6" t="n"/>
+      <c r="G57" s="9" t="n"/>
+      <c r="H57" s="6" t="n"/>
+      <c r="I57" s="6" t="n"/>
+      <c r="J57" s="9" t="n"/>
+      <c r="K57" s="9">
+        <f>IF(OR(I57="",J57=""),"",I57*J57)</f>
+        <v/>
+      </c>
+      <c r="L57" s="7" t="n"/>
+      <c r="M57" s="7" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="n"/>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="7" t="n"/>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="6" t="n"/>
+      <c r="F58" s="6" t="n"/>
+      <c r="G58" s="9" t="n"/>
+      <c r="H58" s="6" t="n"/>
+      <c r="I58" s="6" t="n"/>
+      <c r="J58" s="9" t="n"/>
+      <c r="K58" s="9">
+        <f>IF(OR(I58="",J58=""),"",I58*J58)</f>
+        <v/>
+      </c>
+      <c r="L58" s="7" t="n"/>
+      <c r="M58" s="7" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="n"/>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="7" t="n"/>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="6" t="n"/>
+      <c r="F59" s="6" t="n"/>
+      <c r="G59" s="9" t="n"/>
+      <c r="H59" s="6" t="n"/>
+      <c r="I59" s="6" t="n"/>
+      <c r="J59" s="9" t="n"/>
+      <c r="K59" s="9">
+        <f>IF(OR(I59="",J59=""),"",I59*J59)</f>
+        <v/>
+      </c>
+      <c r="L59" s="7" t="n"/>
+      <c r="M59" s="7" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="n"/>
+      <c r="B60" s="6" t="n"/>
+      <c r="C60" s="7" t="n"/>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="6" t="n"/>
+      <c r="F60" s="6" t="n"/>
+      <c r="G60" s="9" t="n"/>
+      <c r="H60" s="6" t="n"/>
+      <c r="I60" s="6" t="n"/>
+      <c r="J60" s="9" t="n"/>
+      <c r="K60" s="9">
+        <f>IF(OR(I60="",J60=""),"",I60*J60)</f>
+        <v/>
+      </c>
+      <c r="L60" s="7" t="n"/>
+      <c r="M60" s="7" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="n"/>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="7" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="6" t="n"/>
+      <c r="F61" s="6" t="n"/>
+      <c r="G61" s="9" t="n"/>
+      <c r="H61" s="6" t="n"/>
+      <c r="I61" s="6" t="n"/>
+      <c r="J61" s="9" t="n"/>
+      <c r="K61" s="9">
+        <f>IF(OR(I61="",J61=""),"",I61*J61)</f>
+        <v/>
+      </c>
+      <c r="L61" s="7" t="n"/>
+      <c r="M61" s="7" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="8" t="n"/>
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="7" t="n"/>
+      <c r="D62" s="6" t="n"/>
+      <c r="E62" s="6" t="n"/>
+      <c r="F62" s="6" t="n"/>
+      <c r="G62" s="9" t="n"/>
+      <c r="H62" s="6" t="n"/>
+      <c r="I62" s="6" t="n"/>
+      <c r="J62" s="9" t="n"/>
+      <c r="K62" s="9">
+        <f>IF(OR(I62="",J62=""),"",I62*J62)</f>
+        <v/>
+      </c>
+      <c r="L62" s="7" t="n"/>
+      <c r="M62" s="7" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="n"/>
+      <c r="B63" s="6" t="n"/>
+      <c r="C63" s="7" t="n"/>
+      <c r="D63" s="6" t="n"/>
+      <c r="E63" s="6" t="n"/>
+      <c r="F63" s="6" t="n"/>
+      <c r="G63" s="9" t="n"/>
+      <c r="H63" s="6" t="n"/>
+      <c r="I63" s="6" t="n"/>
+      <c r="J63" s="9" t="n"/>
+      <c r="K63" s="9">
+        <f>IF(OR(I63="",J63=""),"",I63*J63)</f>
+        <v/>
+      </c>
+      <c r="L63" s="7" t="n"/>
+      <c r="M63" s="7" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="n"/>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="7" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="6" t="n"/>
+      <c r="F64" s="6" t="n"/>
+      <c r="G64" s="9" t="n"/>
+      <c r="H64" s="6" t="n"/>
+      <c r="I64" s="6" t="n"/>
+      <c r="J64" s="9" t="n"/>
+      <c r="K64" s="9">
+        <f>IF(OR(I64="",J64=""),"",I64*J64)</f>
+        <v/>
+      </c>
+      <c r="L64" s="7" t="n"/>
+      <c r="M64" s="7" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="8" t="n"/>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="7" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="6" t="n"/>
+      <c r="F65" s="6" t="n"/>
+      <c r="G65" s="9" t="n"/>
+      <c r="H65" s="6" t="n"/>
+      <c r="I65" s="6" t="n"/>
+      <c r="J65" s="9" t="n"/>
+      <c r="K65" s="9">
+        <f>IF(OR(I65="",J65=""),"",I65*J65)</f>
+        <v/>
+      </c>
+      <c r="L65" s="7" t="n"/>
+      <c r="M65" s="7" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="n"/>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="7" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
+      <c r="F66" s="6" t="n"/>
+      <c r="G66" s="9" t="n"/>
+      <c r="H66" s="6" t="n"/>
+      <c r="I66" s="6" t="n"/>
+      <c r="J66" s="9" t="n"/>
+      <c r="K66" s="9">
+        <f>IF(OR(I66="",J66=""),"",I66*J66)</f>
+        <v/>
+      </c>
+      <c r="L66" s="7" t="n"/>
+      <c r="M66" s="7" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="8" t="n"/>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="7" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
+      <c r="F67" s="6" t="n"/>
+      <c r="G67" s="9" t="n"/>
+      <c r="H67" s="6" t="n"/>
+      <c r="I67" s="6" t="n"/>
+      <c r="J67" s="9" t="n"/>
+      <c r="K67" s="9">
+        <f>IF(OR(I67="",J67=""),"",I67*J67)</f>
+        <v/>
+      </c>
+      <c r="L67" s="7" t="n"/>
+      <c r="M67" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="H5:M5"/>
+    <mergeCell ref="H4:M4"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B5:E5"/>
+    <mergeCell ref="H2:M2"/>
+    <mergeCell ref="H3:M3"/>
+  </mergeCells>
+  <conditionalFormatting sqref="A8:M67">
+    <cfRule type="expression" priority="1" dxfId="1">
+      <formula>MOD(ROW(),2)=0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="3">
+    <dataValidation sqref="B8:B67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"1st (media roll),2nd,3rd,Attic stock,RFI,Change order"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F8:F67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"8,13"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L8:L67" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Will call,Delivered to site,At Airco warehouse"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Save formula answers so the Tech Filter Form shows in every viewer
openpyxl saves formulas without answers, so Protected View, phone apps,
previews and SharePoint web showed the Tech Filter Form blank. After saving,
write the answers of our simple formulas (copies from the Filter Log and
QTY x unit price) into the file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014FJcz3kiQFukXBXsbksRam
</commit_message>
<xml_diff>
--- a/tracker/templates/TEMPLATE_FilterLog.xlsx
+++ b/tracker/templates/TEMPLATE_FilterLog.xlsx
@@ -2416,7 +2416,7 @@
           <t>Job number</t>
         </is>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="4" t="str">
         <f>IF('Filter Log'!B2="","",'Filter Log'!B2)</f>
         <v/>
       </c>
@@ -2428,7 +2428,7 @@
         </is>
       </c>
       <c r="F2" s="6" t="n"/>
-      <c r="G2" s="4">
+      <c r="G2" s="4" t="str">
         <f>IF('Filter Log'!I2="","",'Filter Log'!I2)</f>
         <v/>
       </c>
@@ -2439,7 +2439,7 @@
           <t>Project name</t>
         </is>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="9" t="str">
         <f>IF('Filter Log'!B3="","",'Filter Log'!B3)</f>
         <v/>
       </c>
@@ -2451,7 +2451,7 @@
         </is>
       </c>
       <c r="F3" s="11" t="n"/>
-      <c r="G3" s="9">
+      <c r="G3" s="9" t="str">
         <f>IF('Filter Log'!I3="","",'Filter Log'!I3)</f>
         <v/>
       </c>
@@ -2462,7 +2462,7 @@
           <t>Phase</t>
         </is>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="9" t="str">
         <f>IF('Filter Log'!B4="","",'Filter Log'!B4)</f>
         <v/>
       </c>
@@ -2474,7 +2474,7 @@
         </is>
       </c>
       <c r="F4" s="11" t="n"/>
-      <c r="G4" s="9">
+      <c r="G4" s="9" t="str">
         <f>IF('Filter Log'!I4="","",'Filter Log'!I4)</f>
         <v/>
       </c>
@@ -2485,7 +2485,7 @@
           <t>Job type</t>
         </is>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="9" t="str">
         <f>IF('Filter Log'!B5="","",'Filter Log'!B5)</f>
         <v/>
       </c>
@@ -2564,23 +2564,23 @@
       </c>
     </row>
     <row r="9" ht="26" customHeight="1">
-      <c r="A9" s="20">
+      <c r="A9" s="20" t="str">
         <f>IF('Filter Log'!A9="","",'Filter Log'!A9)</f>
         <v/>
       </c>
-      <c r="B9" s="21">
+      <c r="B9" s="21" t="str">
         <f>IF('Filter Log'!B9="","",'Filter Log'!B9)</f>
         <v/>
       </c>
-      <c r="C9" s="20">
+      <c r="C9" s="20" t="str">
         <f>IF('Filter Log'!C9="","",'Filter Log'!C9)</f>
         <v/>
       </c>
-      <c r="D9" s="20">
+      <c r="D9" s="20" t="str">
         <f>IF('Filter Log'!D9="","",'Filter Log'!D9)</f>
         <v/>
       </c>
-      <c r="E9" s="20">
+      <c r="E9" s="20" t="str">
         <f>IF('Filter Log'!E9="","",'Filter Log'!E9)</f>
         <v/>
       </c>
@@ -2588,23 +2588,23 @@
       <c r="G9" s="22" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1">
-      <c r="A10" s="20">
+      <c r="A10" s="20" t="str">
         <f>IF('Filter Log'!A10="","",'Filter Log'!A10)</f>
         <v/>
       </c>
-      <c r="B10" s="21">
+      <c r="B10" s="21" t="str">
         <f>IF('Filter Log'!B10="","",'Filter Log'!B10)</f>
         <v/>
       </c>
-      <c r="C10" s="20">
+      <c r="C10" s="20" t="str">
         <f>IF('Filter Log'!C10="","",'Filter Log'!C10)</f>
         <v/>
       </c>
-      <c r="D10" s="20">
+      <c r="D10" s="20" t="str">
         <f>IF('Filter Log'!D10="","",'Filter Log'!D10)</f>
         <v/>
       </c>
-      <c r="E10" s="20">
+      <c r="E10" s="20" t="str">
         <f>IF('Filter Log'!E10="","",'Filter Log'!E10)</f>
         <v/>
       </c>
@@ -2612,23 +2612,23 @@
       <c r="G10" s="22" t="n"/>
     </row>
     <row r="11" ht="26" customHeight="1">
-      <c r="A11" s="20">
+      <c r="A11" s="20" t="str">
         <f>IF('Filter Log'!A11="","",'Filter Log'!A11)</f>
         <v/>
       </c>
-      <c r="B11" s="21">
+      <c r="B11" s="21" t="str">
         <f>IF('Filter Log'!B11="","",'Filter Log'!B11)</f>
         <v/>
       </c>
-      <c r="C11" s="20">
+      <c r="C11" s="20" t="str">
         <f>IF('Filter Log'!C11="","",'Filter Log'!C11)</f>
         <v/>
       </c>
-      <c r="D11" s="20">
+      <c r="D11" s="20" t="str">
         <f>IF('Filter Log'!D11="","",'Filter Log'!D11)</f>
         <v/>
       </c>
-      <c r="E11" s="20">
+      <c r="E11" s="20" t="str">
         <f>IF('Filter Log'!E11="","",'Filter Log'!E11)</f>
         <v/>
       </c>
@@ -2636,23 +2636,23 @@
       <c r="G11" s="22" t="n"/>
     </row>
     <row r="12" ht="26" customHeight="1">
-      <c r="A12" s="20">
+      <c r="A12" s="20" t="str">
         <f>IF('Filter Log'!A12="","",'Filter Log'!A12)</f>
         <v/>
       </c>
-      <c r="B12" s="21">
+      <c r="B12" s="21" t="str">
         <f>IF('Filter Log'!B12="","",'Filter Log'!B12)</f>
         <v/>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="20" t="str">
         <f>IF('Filter Log'!C12="","",'Filter Log'!C12)</f>
         <v/>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="20" t="str">
         <f>IF('Filter Log'!D12="","",'Filter Log'!D12)</f>
         <v/>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="20" t="str">
         <f>IF('Filter Log'!E12="","",'Filter Log'!E12)</f>
         <v/>
       </c>
@@ -2660,23 +2660,23 @@
       <c r="G12" s="22" t="n"/>
     </row>
     <row r="13" ht="26" customHeight="1">
-      <c r="A13" s="20">
+      <c r="A13" s="20" t="str">
         <f>IF('Filter Log'!A13="","",'Filter Log'!A13)</f>
         <v/>
       </c>
-      <c r="B13" s="21">
+      <c r="B13" s="21" t="str">
         <f>IF('Filter Log'!B13="","",'Filter Log'!B13)</f>
         <v/>
       </c>
-      <c r="C13" s="20">
+      <c r="C13" s="20" t="str">
         <f>IF('Filter Log'!C13="","",'Filter Log'!C13)</f>
         <v/>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="20" t="str">
         <f>IF('Filter Log'!D13="","",'Filter Log'!D13)</f>
         <v/>
       </c>
-      <c r="E13" s="20">
+      <c r="E13" s="20" t="str">
         <f>IF('Filter Log'!E13="","",'Filter Log'!E13)</f>
         <v/>
       </c>
@@ -2684,23 +2684,23 @@
       <c r="G13" s="22" t="n"/>
     </row>
     <row r="14" ht="26" customHeight="1">
-      <c r="A14" s="20">
+      <c r="A14" s="20" t="str">
         <f>IF('Filter Log'!A14="","",'Filter Log'!A14)</f>
         <v/>
       </c>
-      <c r="B14" s="21">
+      <c r="B14" s="21" t="str">
         <f>IF('Filter Log'!B14="","",'Filter Log'!B14)</f>
         <v/>
       </c>
-      <c r="C14" s="20">
+      <c r="C14" s="20" t="str">
         <f>IF('Filter Log'!C14="","",'Filter Log'!C14)</f>
         <v/>
       </c>
-      <c r="D14" s="20">
+      <c r="D14" s="20" t="str">
         <f>IF('Filter Log'!D14="","",'Filter Log'!D14)</f>
         <v/>
       </c>
-      <c r="E14" s="20">
+      <c r="E14" s="20" t="str">
         <f>IF('Filter Log'!E14="","",'Filter Log'!E14)</f>
         <v/>
       </c>
@@ -2708,23 +2708,23 @@
       <c r="G14" s="22" t="n"/>
     </row>
     <row r="15" ht="26" customHeight="1">
-      <c r="A15" s="20">
+      <c r="A15" s="20" t="str">
         <f>IF('Filter Log'!A15="","",'Filter Log'!A15)</f>
         <v/>
       </c>
-      <c r="B15" s="21">
+      <c r="B15" s="21" t="str">
         <f>IF('Filter Log'!B15="","",'Filter Log'!B15)</f>
         <v/>
       </c>
-      <c r="C15" s="20">
+      <c r="C15" s="20" t="str">
         <f>IF('Filter Log'!C15="","",'Filter Log'!C15)</f>
         <v/>
       </c>
-      <c r="D15" s="20">
+      <c r="D15" s="20" t="str">
         <f>IF('Filter Log'!D15="","",'Filter Log'!D15)</f>
         <v/>
       </c>
-      <c r="E15" s="20">
+      <c r="E15" s="20" t="str">
         <f>IF('Filter Log'!E15="","",'Filter Log'!E15)</f>
         <v/>
       </c>
@@ -2732,23 +2732,23 @@
       <c r="G15" s="22" t="n"/>
     </row>
     <row r="16" ht="26" customHeight="1">
-      <c r="A16" s="20">
+      <c r="A16" s="20" t="str">
         <f>IF('Filter Log'!A16="","",'Filter Log'!A16)</f>
         <v/>
       </c>
-      <c r="B16" s="21">
+      <c r="B16" s="21" t="str">
         <f>IF('Filter Log'!B16="","",'Filter Log'!B16)</f>
         <v/>
       </c>
-      <c r="C16" s="20">
+      <c r="C16" s="20" t="str">
         <f>IF('Filter Log'!C16="","",'Filter Log'!C16)</f>
         <v/>
       </c>
-      <c r="D16" s="20">
+      <c r="D16" s="20" t="str">
         <f>IF('Filter Log'!D16="","",'Filter Log'!D16)</f>
         <v/>
       </c>
-      <c r="E16" s="20">
+      <c r="E16" s="20" t="str">
         <f>IF('Filter Log'!E16="","",'Filter Log'!E16)</f>
         <v/>
       </c>
@@ -2756,23 +2756,23 @@
       <c r="G16" s="22" t="n"/>
     </row>
     <row r="17" ht="26" customHeight="1">
-      <c r="A17" s="20">
+      <c r="A17" s="20" t="str">
         <f>IF('Filter Log'!A17="","",'Filter Log'!A17)</f>
         <v/>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="21" t="str">
         <f>IF('Filter Log'!B17="","",'Filter Log'!B17)</f>
         <v/>
       </c>
-      <c r="C17" s="20">
+      <c r="C17" s="20" t="str">
         <f>IF('Filter Log'!C17="","",'Filter Log'!C17)</f>
         <v/>
       </c>
-      <c r="D17" s="20">
+      <c r="D17" s="20" t="str">
         <f>IF('Filter Log'!D17="","",'Filter Log'!D17)</f>
         <v/>
       </c>
-      <c r="E17" s="20">
+      <c r="E17" s="20" t="str">
         <f>IF('Filter Log'!E17="","",'Filter Log'!E17)</f>
         <v/>
       </c>
@@ -2780,23 +2780,23 @@
       <c r="G17" s="22" t="n"/>
     </row>
     <row r="18" ht="26" customHeight="1">
-      <c r="A18" s="20">
+      <c r="A18" s="20" t="str">
         <f>IF('Filter Log'!A18="","",'Filter Log'!A18)</f>
         <v/>
       </c>
-      <c r="B18" s="21">
+      <c r="B18" s="21" t="str">
         <f>IF('Filter Log'!B18="","",'Filter Log'!B18)</f>
         <v/>
       </c>
-      <c r="C18" s="20">
+      <c r="C18" s="20" t="str">
         <f>IF('Filter Log'!C18="","",'Filter Log'!C18)</f>
         <v/>
       </c>
-      <c r="D18" s="20">
+      <c r="D18" s="20" t="str">
         <f>IF('Filter Log'!D18="","",'Filter Log'!D18)</f>
         <v/>
       </c>
-      <c r="E18" s="20">
+      <c r="E18" s="20" t="str">
         <f>IF('Filter Log'!E18="","",'Filter Log'!E18)</f>
         <v/>
       </c>
@@ -2804,23 +2804,23 @@
       <c r="G18" s="22" t="n"/>
     </row>
     <row r="19" ht="26" customHeight="1">
-      <c r="A19" s="20">
+      <c r="A19" s="20" t="str">
         <f>IF('Filter Log'!A19="","",'Filter Log'!A19)</f>
         <v/>
       </c>
-      <c r="B19" s="21">
+      <c r="B19" s="21" t="str">
         <f>IF('Filter Log'!B19="","",'Filter Log'!B19)</f>
         <v/>
       </c>
-      <c r="C19" s="20">
+      <c r="C19" s="20" t="str">
         <f>IF('Filter Log'!C19="","",'Filter Log'!C19)</f>
         <v/>
       </c>
-      <c r="D19" s="20">
+      <c r="D19" s="20" t="str">
         <f>IF('Filter Log'!D19="","",'Filter Log'!D19)</f>
         <v/>
       </c>
-      <c r="E19" s="20">
+      <c r="E19" s="20" t="str">
         <f>IF('Filter Log'!E19="","",'Filter Log'!E19)</f>
         <v/>
       </c>
@@ -2828,23 +2828,23 @@
       <c r="G19" s="22" t="n"/>
     </row>
     <row r="20" ht="26" customHeight="1">
-      <c r="A20" s="20">
+      <c r="A20" s="20" t="str">
         <f>IF('Filter Log'!A20="","",'Filter Log'!A20)</f>
         <v/>
       </c>
-      <c r="B20" s="21">
+      <c r="B20" s="21" t="str">
         <f>IF('Filter Log'!B20="","",'Filter Log'!B20)</f>
         <v/>
       </c>
-      <c r="C20" s="20">
+      <c r="C20" s="20" t="str">
         <f>IF('Filter Log'!C20="","",'Filter Log'!C20)</f>
         <v/>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="20" t="str">
         <f>IF('Filter Log'!D20="","",'Filter Log'!D20)</f>
         <v/>
       </c>
-      <c r="E20" s="20">
+      <c r="E20" s="20" t="str">
         <f>IF('Filter Log'!E20="","",'Filter Log'!E20)</f>
         <v/>
       </c>
@@ -2852,23 +2852,23 @@
       <c r="G20" s="22" t="n"/>
     </row>
     <row r="21" ht="26" customHeight="1">
-      <c r="A21" s="20">
+      <c r="A21" s="20" t="str">
         <f>IF('Filter Log'!A21="","",'Filter Log'!A21)</f>
         <v/>
       </c>
-      <c r="B21" s="21">
+      <c r="B21" s="21" t="str">
         <f>IF('Filter Log'!B21="","",'Filter Log'!B21)</f>
         <v/>
       </c>
-      <c r="C21" s="20">
+      <c r="C21" s="20" t="str">
         <f>IF('Filter Log'!C21="","",'Filter Log'!C21)</f>
         <v/>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="20" t="str">
         <f>IF('Filter Log'!D21="","",'Filter Log'!D21)</f>
         <v/>
       </c>
-      <c r="E21" s="20">
+      <c r="E21" s="20" t="str">
         <f>IF('Filter Log'!E21="","",'Filter Log'!E21)</f>
         <v/>
       </c>
@@ -2876,23 +2876,23 @@
       <c r="G21" s="22" t="n"/>
     </row>
     <row r="22" ht="26" customHeight="1">
-      <c r="A22" s="20">
+      <c r="A22" s="20" t="str">
         <f>IF('Filter Log'!A22="","",'Filter Log'!A22)</f>
         <v/>
       </c>
-      <c r="B22" s="21">
+      <c r="B22" s="21" t="str">
         <f>IF('Filter Log'!B22="","",'Filter Log'!B22)</f>
         <v/>
       </c>
-      <c r="C22" s="20">
+      <c r="C22" s="20" t="str">
         <f>IF('Filter Log'!C22="","",'Filter Log'!C22)</f>
         <v/>
       </c>
-      <c r="D22" s="20">
+      <c r="D22" s="20" t="str">
         <f>IF('Filter Log'!D22="","",'Filter Log'!D22)</f>
         <v/>
       </c>
-      <c r="E22" s="20">
+      <c r="E22" s="20" t="str">
         <f>IF('Filter Log'!E22="","",'Filter Log'!E22)</f>
         <v/>
       </c>
@@ -2900,23 +2900,23 @@
       <c r="G22" s="22" t="n"/>
     </row>
     <row r="23" ht="26" customHeight="1">
-      <c r="A23" s="20">
+      <c r="A23" s="20" t="str">
         <f>IF('Filter Log'!A23="","",'Filter Log'!A23)</f>
         <v/>
       </c>
-      <c r="B23" s="21">
+      <c r="B23" s="21" t="str">
         <f>IF('Filter Log'!B23="","",'Filter Log'!B23)</f>
         <v/>
       </c>
-      <c r="C23" s="20">
+      <c r="C23" s="20" t="str">
         <f>IF('Filter Log'!C23="","",'Filter Log'!C23)</f>
         <v/>
       </c>
-      <c r="D23" s="20">
+      <c r="D23" s="20" t="str">
         <f>IF('Filter Log'!D23="","",'Filter Log'!D23)</f>
         <v/>
       </c>
-      <c r="E23" s="20">
+      <c r="E23" s="20" t="str">
         <f>IF('Filter Log'!E23="","",'Filter Log'!E23)</f>
         <v/>
       </c>
@@ -2924,23 +2924,23 @@
       <c r="G23" s="22" t="n"/>
     </row>
     <row r="24" ht="26" customHeight="1">
-      <c r="A24" s="20">
+      <c r="A24" s="20" t="str">
         <f>IF('Filter Log'!A24="","",'Filter Log'!A24)</f>
         <v/>
       </c>
-      <c r="B24" s="21">
+      <c r="B24" s="21" t="str">
         <f>IF('Filter Log'!B24="","",'Filter Log'!B24)</f>
         <v/>
       </c>
-      <c r="C24" s="20">
+      <c r="C24" s="20" t="str">
         <f>IF('Filter Log'!C24="","",'Filter Log'!C24)</f>
         <v/>
       </c>
-      <c r="D24" s="20">
+      <c r="D24" s="20" t="str">
         <f>IF('Filter Log'!D24="","",'Filter Log'!D24)</f>
         <v/>
       </c>
-      <c r="E24" s="20">
+      <c r="E24" s="20" t="str">
         <f>IF('Filter Log'!E24="","",'Filter Log'!E24)</f>
         <v/>
       </c>
@@ -2948,23 +2948,23 @@
       <c r="G24" s="22" t="n"/>
     </row>
     <row r="25" ht="26" customHeight="1">
-      <c r="A25" s="20">
+      <c r="A25" s="20" t="str">
         <f>IF('Filter Log'!A25="","",'Filter Log'!A25)</f>
         <v/>
       </c>
-      <c r="B25" s="21">
+      <c r="B25" s="21" t="str">
         <f>IF('Filter Log'!B25="","",'Filter Log'!B25)</f>
         <v/>
       </c>
-      <c r="C25" s="20">
+      <c r="C25" s="20" t="str">
         <f>IF('Filter Log'!C25="","",'Filter Log'!C25)</f>
         <v/>
       </c>
-      <c r="D25" s="20">
+      <c r="D25" s="20" t="str">
         <f>IF('Filter Log'!D25="","",'Filter Log'!D25)</f>
         <v/>
       </c>
-      <c r="E25" s="20">
+      <c r="E25" s="20" t="str">
         <f>IF('Filter Log'!E25="","",'Filter Log'!E25)</f>
         <v/>
       </c>
@@ -2972,23 +2972,23 @@
       <c r="G25" s="22" t="n"/>
     </row>
     <row r="26" ht="26" customHeight="1">
-      <c r="A26" s="20">
+      <c r="A26" s="20" t="str">
         <f>IF('Filter Log'!A26="","",'Filter Log'!A26)</f>
         <v/>
       </c>
-      <c r="B26" s="21">
+      <c r="B26" s="21" t="str">
         <f>IF('Filter Log'!B26="","",'Filter Log'!B26)</f>
         <v/>
       </c>
-      <c r="C26" s="20">
+      <c r="C26" s="20" t="str">
         <f>IF('Filter Log'!C26="","",'Filter Log'!C26)</f>
         <v/>
       </c>
-      <c r="D26" s="20">
+      <c r="D26" s="20" t="str">
         <f>IF('Filter Log'!D26="","",'Filter Log'!D26)</f>
         <v/>
       </c>
-      <c r="E26" s="20">
+      <c r="E26" s="20" t="str">
         <f>IF('Filter Log'!E26="","",'Filter Log'!E26)</f>
         <v/>
       </c>
@@ -2996,23 +2996,23 @@
       <c r="G26" s="22" t="n"/>
     </row>
     <row r="27" ht="26" customHeight="1">
-      <c r="A27" s="20">
+      <c r="A27" s="20" t="str">
         <f>IF('Filter Log'!A27="","",'Filter Log'!A27)</f>
         <v/>
       </c>
-      <c r="B27" s="21">
+      <c r="B27" s="21" t="str">
         <f>IF('Filter Log'!B27="","",'Filter Log'!B27)</f>
         <v/>
       </c>
-      <c r="C27" s="20">
+      <c r="C27" s="20" t="str">
         <f>IF('Filter Log'!C27="","",'Filter Log'!C27)</f>
         <v/>
       </c>
-      <c r="D27" s="20">
+      <c r="D27" s="20" t="str">
         <f>IF('Filter Log'!D27="","",'Filter Log'!D27)</f>
         <v/>
       </c>
-      <c r="E27" s="20">
+      <c r="E27" s="20" t="str">
         <f>IF('Filter Log'!E27="","",'Filter Log'!E27)</f>
         <v/>
       </c>
@@ -3020,23 +3020,23 @@
       <c r="G27" s="22" t="n"/>
     </row>
     <row r="28" ht="26" customHeight="1">
-      <c r="A28" s="20">
+      <c r="A28" s="20" t="str">
         <f>IF('Filter Log'!A28="","",'Filter Log'!A28)</f>
         <v/>
       </c>
-      <c r="B28" s="21">
+      <c r="B28" s="21" t="str">
         <f>IF('Filter Log'!B28="","",'Filter Log'!B28)</f>
         <v/>
       </c>
-      <c r="C28" s="20">
+      <c r="C28" s="20" t="str">
         <f>IF('Filter Log'!C28="","",'Filter Log'!C28)</f>
         <v/>
       </c>
-      <c r="D28" s="20">
+      <c r="D28" s="20" t="str">
         <f>IF('Filter Log'!D28="","",'Filter Log'!D28)</f>
         <v/>
       </c>
-      <c r="E28" s="20">
+      <c r="E28" s="20" t="str">
         <f>IF('Filter Log'!E28="","",'Filter Log'!E28)</f>
         <v/>
       </c>
@@ -3044,23 +3044,23 @@
       <c r="G28" s="22" t="n"/>
     </row>
     <row r="29" ht="26" customHeight="1">
-      <c r="A29" s="20">
+      <c r="A29" s="20" t="str">
         <f>IF('Filter Log'!A29="","",'Filter Log'!A29)</f>
         <v/>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="21" t="str">
         <f>IF('Filter Log'!B29="","",'Filter Log'!B29)</f>
         <v/>
       </c>
-      <c r="C29" s="20">
+      <c r="C29" s="20" t="str">
         <f>IF('Filter Log'!C29="","",'Filter Log'!C29)</f>
         <v/>
       </c>
-      <c r="D29" s="20">
+      <c r="D29" s="20" t="str">
         <f>IF('Filter Log'!D29="","",'Filter Log'!D29)</f>
         <v/>
       </c>
-      <c r="E29" s="20">
+      <c r="E29" s="20" t="str">
         <f>IF('Filter Log'!E29="","",'Filter Log'!E29)</f>
         <v/>
       </c>
@@ -3068,23 +3068,23 @@
       <c r="G29" s="22" t="n"/>
     </row>
     <row r="30" ht="26" customHeight="1">
-      <c r="A30" s="20">
+      <c r="A30" s="20" t="str">
         <f>IF('Filter Log'!A30="","",'Filter Log'!A30)</f>
         <v/>
       </c>
-      <c r="B30" s="21">
+      <c r="B30" s="21" t="str">
         <f>IF('Filter Log'!B30="","",'Filter Log'!B30)</f>
         <v/>
       </c>
-      <c r="C30" s="20">
+      <c r="C30" s="20" t="str">
         <f>IF('Filter Log'!C30="","",'Filter Log'!C30)</f>
         <v/>
       </c>
-      <c r="D30" s="20">
+      <c r="D30" s="20" t="str">
         <f>IF('Filter Log'!D30="","",'Filter Log'!D30)</f>
         <v/>
       </c>
-      <c r="E30" s="20">
+      <c r="E30" s="20" t="str">
         <f>IF('Filter Log'!E30="","",'Filter Log'!E30)</f>
         <v/>
       </c>
@@ -3092,23 +3092,23 @@
       <c r="G30" s="22" t="n"/>
     </row>
     <row r="31" ht="26" customHeight="1">
-      <c r="A31" s="20">
+      <c r="A31" s="20" t="str">
         <f>IF('Filter Log'!A31="","",'Filter Log'!A31)</f>
         <v/>
       </c>
-      <c r="B31" s="21">
+      <c r="B31" s="21" t="str">
         <f>IF('Filter Log'!B31="","",'Filter Log'!B31)</f>
         <v/>
       </c>
-      <c r="C31" s="20">
+      <c r="C31" s="20" t="str">
         <f>IF('Filter Log'!C31="","",'Filter Log'!C31)</f>
         <v/>
       </c>
-      <c r="D31" s="20">
+      <c r="D31" s="20" t="str">
         <f>IF('Filter Log'!D31="","",'Filter Log'!D31)</f>
         <v/>
       </c>
-      <c r="E31" s="20">
+      <c r="E31" s="20" t="str">
         <f>IF('Filter Log'!E31="","",'Filter Log'!E31)</f>
         <v/>
       </c>
@@ -3116,23 +3116,23 @@
       <c r="G31" s="22" t="n"/>
     </row>
     <row r="32" ht="26" customHeight="1">
-      <c r="A32" s="20">
+      <c r="A32" s="20" t="str">
         <f>IF('Filter Log'!A32="","",'Filter Log'!A32)</f>
         <v/>
       </c>
-      <c r="B32" s="21">
+      <c r="B32" s="21" t="str">
         <f>IF('Filter Log'!B32="","",'Filter Log'!B32)</f>
         <v/>
       </c>
-      <c r="C32" s="20">
+      <c r="C32" s="20" t="str">
         <f>IF('Filter Log'!C32="","",'Filter Log'!C32)</f>
         <v/>
       </c>
-      <c r="D32" s="20">
+      <c r="D32" s="20" t="str">
         <f>IF('Filter Log'!D32="","",'Filter Log'!D32)</f>
         <v/>
       </c>
-      <c r="E32" s="20">
+      <c r="E32" s="20" t="str">
         <f>IF('Filter Log'!E32="","",'Filter Log'!E32)</f>
         <v/>
       </c>
@@ -3140,23 +3140,23 @@
       <c r="G32" s="22" t="n"/>
     </row>
     <row r="33" ht="26" customHeight="1">
-      <c r="A33" s="20">
+      <c r="A33" s="20" t="str">
         <f>IF('Filter Log'!A33="","",'Filter Log'!A33)</f>
         <v/>
       </c>
-      <c r="B33" s="21">
+      <c r="B33" s="21" t="str">
         <f>IF('Filter Log'!B33="","",'Filter Log'!B33)</f>
         <v/>
       </c>
-      <c r="C33" s="20">
+      <c r="C33" s="20" t="str">
         <f>IF('Filter Log'!C33="","",'Filter Log'!C33)</f>
         <v/>
       </c>
-      <c r="D33" s="20">
+      <c r="D33" s="20" t="str">
         <f>IF('Filter Log'!D33="","",'Filter Log'!D33)</f>
         <v/>
       </c>
-      <c r="E33" s="20">
+      <c r="E33" s="20" t="str">
         <f>IF('Filter Log'!E33="","",'Filter Log'!E33)</f>
         <v/>
       </c>
@@ -3164,23 +3164,23 @@
       <c r="G33" s="22" t="n"/>
     </row>
     <row r="34" ht="26" customHeight="1">
-      <c r="A34" s="20">
+      <c r="A34" s="20" t="str">
         <f>IF('Filter Log'!A34="","",'Filter Log'!A34)</f>
         <v/>
       </c>
-      <c r="B34" s="21">
+      <c r="B34" s="21" t="str">
         <f>IF('Filter Log'!B34="","",'Filter Log'!B34)</f>
         <v/>
       </c>
-      <c r="C34" s="20">
+      <c r="C34" s="20" t="str">
         <f>IF('Filter Log'!C34="","",'Filter Log'!C34)</f>
         <v/>
       </c>
-      <c r="D34" s="20">
+      <c r="D34" s="20" t="str">
         <f>IF('Filter Log'!D34="","",'Filter Log'!D34)</f>
         <v/>
       </c>
-      <c r="E34" s="20">
+      <c r="E34" s="20" t="str">
         <f>IF('Filter Log'!E34="","",'Filter Log'!E34)</f>
         <v/>
       </c>
@@ -3188,23 +3188,23 @@
       <c r="G34" s="22" t="n"/>
     </row>
     <row r="35" ht="26" customHeight="1">
-      <c r="A35" s="20">
+      <c r="A35" s="20" t="str">
         <f>IF('Filter Log'!A35="","",'Filter Log'!A35)</f>
         <v/>
       </c>
-      <c r="B35" s="21">
+      <c r="B35" s="21" t="str">
         <f>IF('Filter Log'!B35="","",'Filter Log'!B35)</f>
         <v/>
       </c>
-      <c r="C35" s="20">
+      <c r="C35" s="20" t="str">
         <f>IF('Filter Log'!C35="","",'Filter Log'!C35)</f>
         <v/>
       </c>
-      <c r="D35" s="20">
+      <c r="D35" s="20" t="str">
         <f>IF('Filter Log'!D35="","",'Filter Log'!D35)</f>
         <v/>
       </c>
-      <c r="E35" s="20">
+      <c r="E35" s="20" t="str">
         <f>IF('Filter Log'!E35="","",'Filter Log'!E35)</f>
         <v/>
       </c>
@@ -3212,23 +3212,23 @@
       <c r="G35" s="22" t="n"/>
     </row>
     <row r="36" ht="26" customHeight="1">
-      <c r="A36" s="20">
+      <c r="A36" s="20" t="str">
         <f>IF('Filter Log'!A36="","",'Filter Log'!A36)</f>
         <v/>
       </c>
-      <c r="B36" s="21">
+      <c r="B36" s="21" t="str">
         <f>IF('Filter Log'!B36="","",'Filter Log'!B36)</f>
         <v/>
       </c>
-      <c r="C36" s="20">
+      <c r="C36" s="20" t="str">
         <f>IF('Filter Log'!C36="","",'Filter Log'!C36)</f>
         <v/>
       </c>
-      <c r="D36" s="20">
+      <c r="D36" s="20" t="str">
         <f>IF('Filter Log'!D36="","",'Filter Log'!D36)</f>
         <v/>
       </c>
-      <c r="E36" s="20">
+      <c r="E36" s="20" t="str">
         <f>IF('Filter Log'!E36="","",'Filter Log'!E36)</f>
         <v/>
       </c>
@@ -3236,23 +3236,23 @@
       <c r="G36" s="22" t="n"/>
     </row>
     <row r="37" ht="26" customHeight="1">
-      <c r="A37" s="20">
+      <c r="A37" s="20" t="str">
         <f>IF('Filter Log'!A37="","",'Filter Log'!A37)</f>
         <v/>
       </c>
-      <c r="B37" s="21">
+      <c r="B37" s="21" t="str">
         <f>IF('Filter Log'!B37="","",'Filter Log'!B37)</f>
         <v/>
       </c>
-      <c r="C37" s="20">
+      <c r="C37" s="20" t="str">
         <f>IF('Filter Log'!C37="","",'Filter Log'!C37)</f>
         <v/>
       </c>
-      <c r="D37" s="20">
+      <c r="D37" s="20" t="str">
         <f>IF('Filter Log'!D37="","",'Filter Log'!D37)</f>
         <v/>
       </c>
-      <c r="E37" s="20">
+      <c r="E37" s="20" t="str">
         <f>IF('Filter Log'!E37="","",'Filter Log'!E37)</f>
         <v/>
       </c>
@@ -3260,23 +3260,23 @@
       <c r="G37" s="22" t="n"/>
     </row>
     <row r="38" ht="26" customHeight="1">
-      <c r="A38" s="20">
+      <c r="A38" s="20" t="str">
         <f>IF('Filter Log'!A38="","",'Filter Log'!A38)</f>
         <v/>
       </c>
-      <c r="B38" s="21">
+      <c r="B38" s="21" t="str">
         <f>IF('Filter Log'!B38="","",'Filter Log'!B38)</f>
         <v/>
       </c>
-      <c r="C38" s="20">
+      <c r="C38" s="20" t="str">
         <f>IF('Filter Log'!C38="","",'Filter Log'!C38)</f>
         <v/>
       </c>
-      <c r="D38" s="20">
+      <c r="D38" s="20" t="str">
         <f>IF('Filter Log'!D38="","",'Filter Log'!D38)</f>
         <v/>
       </c>
-      <c r="E38" s="20">
+      <c r="E38" s="20" t="str">
         <f>IF('Filter Log'!E38="","",'Filter Log'!E38)</f>
         <v/>
       </c>
@@ -3284,23 +3284,23 @@
       <c r="G38" s="22" t="n"/>
     </row>
     <row r="39" ht="26" customHeight="1">
-      <c r="A39" s="20">
+      <c r="A39" s="20" t="str">
         <f>IF('Filter Log'!A39="","",'Filter Log'!A39)</f>
         <v/>
       </c>
-      <c r="B39" s="21">
+      <c r="B39" s="21" t="str">
         <f>IF('Filter Log'!B39="","",'Filter Log'!B39)</f>
         <v/>
       </c>
-      <c r="C39" s="20">
+      <c r="C39" s="20" t="str">
         <f>IF('Filter Log'!C39="","",'Filter Log'!C39)</f>
         <v/>
       </c>
-      <c r="D39" s="20">
+      <c r="D39" s="20" t="str">
         <f>IF('Filter Log'!D39="","",'Filter Log'!D39)</f>
         <v/>
       </c>
-      <c r="E39" s="20">
+      <c r="E39" s="20" t="str">
         <f>IF('Filter Log'!E39="","",'Filter Log'!E39)</f>
         <v/>
       </c>
@@ -3308,23 +3308,23 @@
       <c r="G39" s="22" t="n"/>
     </row>
     <row r="40" ht="26" customHeight="1">
-      <c r="A40" s="20">
+      <c r="A40" s="20" t="str">
         <f>IF('Filter Log'!A40="","",'Filter Log'!A40)</f>
         <v/>
       </c>
-      <c r="B40" s="21">
+      <c r="B40" s="21" t="str">
         <f>IF('Filter Log'!B40="","",'Filter Log'!B40)</f>
         <v/>
       </c>
-      <c r="C40" s="20">
+      <c r="C40" s="20" t="str">
         <f>IF('Filter Log'!C40="","",'Filter Log'!C40)</f>
         <v/>
       </c>
-      <c r="D40" s="20">
+      <c r="D40" s="20" t="str">
         <f>IF('Filter Log'!D40="","",'Filter Log'!D40)</f>
         <v/>
       </c>
-      <c r="E40" s="20">
+      <c r="E40" s="20" t="str">
         <f>IF('Filter Log'!E40="","",'Filter Log'!E40)</f>
         <v/>
       </c>
@@ -3332,23 +3332,23 @@
       <c r="G40" s="22" t="n"/>
     </row>
     <row r="41" ht="26" customHeight="1">
-      <c r="A41" s="20">
+      <c r="A41" s="20" t="str">
         <f>IF('Filter Log'!A41="","",'Filter Log'!A41)</f>
         <v/>
       </c>
-      <c r="B41" s="21">
+      <c r="B41" s="21" t="str">
         <f>IF('Filter Log'!B41="","",'Filter Log'!B41)</f>
         <v/>
       </c>
-      <c r="C41" s="20">
+      <c r="C41" s="20" t="str">
         <f>IF('Filter Log'!C41="","",'Filter Log'!C41)</f>
         <v/>
       </c>
-      <c r="D41" s="20">
+      <c r="D41" s="20" t="str">
         <f>IF('Filter Log'!D41="","",'Filter Log'!D41)</f>
         <v/>
       </c>
-      <c r="E41" s="20">
+      <c r="E41" s="20" t="str">
         <f>IF('Filter Log'!E41="","",'Filter Log'!E41)</f>
         <v/>
       </c>
@@ -3356,23 +3356,23 @@
       <c r="G41" s="22" t="n"/>
     </row>
     <row r="42" ht="26" customHeight="1">
-      <c r="A42" s="20">
+      <c r="A42" s="20" t="str">
         <f>IF('Filter Log'!A42="","",'Filter Log'!A42)</f>
         <v/>
       </c>
-      <c r="B42" s="21">
+      <c r="B42" s="21" t="str">
         <f>IF('Filter Log'!B42="","",'Filter Log'!B42)</f>
         <v/>
       </c>
-      <c r="C42" s="20">
+      <c r="C42" s="20" t="str">
         <f>IF('Filter Log'!C42="","",'Filter Log'!C42)</f>
         <v/>
       </c>
-      <c r="D42" s="20">
+      <c r="D42" s="20" t="str">
         <f>IF('Filter Log'!D42="","",'Filter Log'!D42)</f>
         <v/>
       </c>
-      <c r="E42" s="20">
+      <c r="E42" s="20" t="str">
         <f>IF('Filter Log'!E42="","",'Filter Log'!E42)</f>
         <v/>
       </c>
@@ -3380,23 +3380,23 @@
       <c r="G42" s="22" t="n"/>
     </row>
     <row r="43" ht="26" customHeight="1">
-      <c r="A43" s="20">
+      <c r="A43" s="20" t="str">
         <f>IF('Filter Log'!A43="","",'Filter Log'!A43)</f>
         <v/>
       </c>
-      <c r="B43" s="21">
+      <c r="B43" s="21" t="str">
         <f>IF('Filter Log'!B43="","",'Filter Log'!B43)</f>
         <v/>
       </c>
-      <c r="C43" s="20">
+      <c r="C43" s="20" t="str">
         <f>IF('Filter Log'!C43="","",'Filter Log'!C43)</f>
         <v/>
       </c>
-      <c r="D43" s="20">
+      <c r="D43" s="20" t="str">
         <f>IF('Filter Log'!D43="","",'Filter Log'!D43)</f>
         <v/>
       </c>
-      <c r="E43" s="20">
+      <c r="E43" s="20" t="str">
         <f>IF('Filter Log'!E43="","",'Filter Log'!E43)</f>
         <v/>
       </c>
@@ -3404,23 +3404,23 @@
       <c r="G43" s="22" t="n"/>
     </row>
     <row r="44" ht="26" customHeight="1">
-      <c r="A44" s="20">
+      <c r="A44" s="20" t="str">
         <f>IF('Filter Log'!A44="","",'Filter Log'!A44)</f>
         <v/>
       </c>
-      <c r="B44" s="21">
+      <c r="B44" s="21" t="str">
         <f>IF('Filter Log'!B44="","",'Filter Log'!B44)</f>
         <v/>
       </c>
-      <c r="C44" s="20">
+      <c r="C44" s="20" t="str">
         <f>IF('Filter Log'!C44="","",'Filter Log'!C44)</f>
         <v/>
       </c>
-      <c r="D44" s="20">
+      <c r="D44" s="20" t="str">
         <f>IF('Filter Log'!D44="","",'Filter Log'!D44)</f>
         <v/>
       </c>
-      <c r="E44" s="20">
+      <c r="E44" s="20" t="str">
         <f>IF('Filter Log'!E44="","",'Filter Log'!E44)</f>
         <v/>
       </c>
@@ -3428,23 +3428,23 @@
       <c r="G44" s="22" t="n"/>
     </row>
     <row r="45" ht="26" customHeight="1">
-      <c r="A45" s="20">
+      <c r="A45" s="20" t="str">
         <f>IF('Filter Log'!A45="","",'Filter Log'!A45)</f>
         <v/>
       </c>
-      <c r="B45" s="21">
+      <c r="B45" s="21" t="str">
         <f>IF('Filter Log'!B45="","",'Filter Log'!B45)</f>
         <v/>
       </c>
-      <c r="C45" s="20">
+      <c r="C45" s="20" t="str">
         <f>IF('Filter Log'!C45="","",'Filter Log'!C45)</f>
         <v/>
       </c>
-      <c r="D45" s="20">
+      <c r="D45" s="20" t="str">
         <f>IF('Filter Log'!D45="","",'Filter Log'!D45)</f>
         <v/>
       </c>
-      <c r="E45" s="20">
+      <c r="E45" s="20" t="str">
         <f>IF('Filter Log'!E45="","",'Filter Log'!E45)</f>
         <v/>
       </c>
@@ -3452,23 +3452,23 @@
       <c r="G45" s="22" t="n"/>
     </row>
     <row r="46" ht="26" customHeight="1">
-      <c r="A46" s="20">
+      <c r="A46" s="20" t="str">
         <f>IF('Filter Log'!A46="","",'Filter Log'!A46)</f>
         <v/>
       </c>
-      <c r="B46" s="21">
+      <c r="B46" s="21" t="str">
         <f>IF('Filter Log'!B46="","",'Filter Log'!B46)</f>
         <v/>
       </c>
-      <c r="C46" s="20">
+      <c r="C46" s="20" t="str">
         <f>IF('Filter Log'!C46="","",'Filter Log'!C46)</f>
         <v/>
       </c>
-      <c r="D46" s="20">
+      <c r="D46" s="20" t="str">
         <f>IF('Filter Log'!D46="","",'Filter Log'!D46)</f>
         <v/>
       </c>
-      <c r="E46" s="20">
+      <c r="E46" s="20" t="str">
         <f>IF('Filter Log'!E46="","",'Filter Log'!E46)</f>
         <v/>
       </c>
@@ -3476,23 +3476,23 @@
       <c r="G46" s="22" t="n"/>
     </row>
     <row r="47" ht="26" customHeight="1">
-      <c r="A47" s="20">
+      <c r="A47" s="20" t="str">
         <f>IF('Filter Log'!A47="","",'Filter Log'!A47)</f>
         <v/>
       </c>
-      <c r="B47" s="21">
+      <c r="B47" s="21" t="str">
         <f>IF('Filter Log'!B47="","",'Filter Log'!B47)</f>
         <v/>
       </c>
-      <c r="C47" s="20">
+      <c r="C47" s="20" t="str">
         <f>IF('Filter Log'!C47="","",'Filter Log'!C47)</f>
         <v/>
       </c>
-      <c r="D47" s="20">
+      <c r="D47" s="20" t="str">
         <f>IF('Filter Log'!D47="","",'Filter Log'!D47)</f>
         <v/>
       </c>
-      <c r="E47" s="20">
+      <c r="E47" s="20" t="str">
         <f>IF('Filter Log'!E47="","",'Filter Log'!E47)</f>
         <v/>
       </c>
@@ -3500,23 +3500,23 @@
       <c r="G47" s="22" t="n"/>
     </row>
     <row r="48" ht="26" customHeight="1">
-      <c r="A48" s="20">
+      <c r="A48" s="20" t="str">
         <f>IF('Filter Log'!A48="","",'Filter Log'!A48)</f>
         <v/>
       </c>
-      <c r="B48" s="21">
+      <c r="B48" s="21" t="str">
         <f>IF('Filter Log'!B48="","",'Filter Log'!B48)</f>
         <v/>
       </c>
-      <c r="C48" s="20">
+      <c r="C48" s="20" t="str">
         <f>IF('Filter Log'!C48="","",'Filter Log'!C48)</f>
         <v/>
       </c>
-      <c r="D48" s="20">
+      <c r="D48" s="20" t="str">
         <f>IF('Filter Log'!D48="","",'Filter Log'!D48)</f>
         <v/>
       </c>
-      <c r="E48" s="20">
+      <c r="E48" s="20" t="str">
         <f>IF('Filter Log'!E48="","",'Filter Log'!E48)</f>
         <v/>
       </c>
@@ -3524,23 +3524,23 @@
       <c r="G48" s="22" t="n"/>
     </row>
     <row r="49" ht="26" customHeight="1">
-      <c r="A49" s="20">
+      <c r="A49" s="20" t="str">
         <f>IF('Filter Log'!A49="","",'Filter Log'!A49)</f>
         <v/>
       </c>
-      <c r="B49" s="21">
+      <c r="B49" s="21" t="str">
         <f>IF('Filter Log'!B49="","",'Filter Log'!B49)</f>
         <v/>
       </c>
-      <c r="C49" s="20">
+      <c r="C49" s="20" t="str">
         <f>IF('Filter Log'!C49="","",'Filter Log'!C49)</f>
         <v/>
       </c>
-      <c r="D49" s="20">
+      <c r="D49" s="20" t="str">
         <f>IF('Filter Log'!D49="","",'Filter Log'!D49)</f>
         <v/>
       </c>
-      <c r="E49" s="20">
+      <c r="E49" s="20" t="str">
         <f>IF('Filter Log'!E49="","",'Filter Log'!E49)</f>
         <v/>
       </c>
@@ -3548,23 +3548,23 @@
       <c r="G49" s="22" t="n"/>
     </row>
     <row r="50" ht="26" customHeight="1">
-      <c r="A50" s="20">
+      <c r="A50" s="20" t="str">
         <f>IF('Filter Log'!A50="","",'Filter Log'!A50)</f>
         <v/>
       </c>
-      <c r="B50" s="21">
+      <c r="B50" s="21" t="str">
         <f>IF('Filter Log'!B50="","",'Filter Log'!B50)</f>
         <v/>
       </c>
-      <c r="C50" s="20">
+      <c r="C50" s="20" t="str">
         <f>IF('Filter Log'!C50="","",'Filter Log'!C50)</f>
         <v/>
       </c>
-      <c r="D50" s="20">
+      <c r="D50" s="20" t="str">
         <f>IF('Filter Log'!D50="","",'Filter Log'!D50)</f>
         <v/>
       </c>
-      <c r="E50" s="20">
+      <c r="E50" s="20" t="str">
         <f>IF('Filter Log'!E50="","",'Filter Log'!E50)</f>
         <v/>
       </c>
@@ -3572,23 +3572,23 @@
       <c r="G50" s="22" t="n"/>
     </row>
     <row r="51" ht="26" customHeight="1">
-      <c r="A51" s="20">
+      <c r="A51" s="20" t="str">
         <f>IF('Filter Log'!A51="","",'Filter Log'!A51)</f>
         <v/>
       </c>
-      <c r="B51" s="21">
+      <c r="B51" s="21" t="str">
         <f>IF('Filter Log'!B51="","",'Filter Log'!B51)</f>
         <v/>
       </c>
-      <c r="C51" s="20">
+      <c r="C51" s="20" t="str">
         <f>IF('Filter Log'!C51="","",'Filter Log'!C51)</f>
         <v/>
       </c>
-      <c r="D51" s="20">
+      <c r="D51" s="20" t="str">
         <f>IF('Filter Log'!D51="","",'Filter Log'!D51)</f>
         <v/>
       </c>
-      <c r="E51" s="20">
+      <c r="E51" s="20" t="str">
         <f>IF('Filter Log'!E51="","",'Filter Log'!E51)</f>
         <v/>
       </c>
@@ -3596,23 +3596,23 @@
       <c r="G51" s="22" t="n"/>
     </row>
     <row r="52" ht="26" customHeight="1">
-      <c r="A52" s="20">
+      <c r="A52" s="20" t="str">
         <f>IF('Filter Log'!A52="","",'Filter Log'!A52)</f>
         <v/>
       </c>
-      <c r="B52" s="21">
+      <c r="B52" s="21" t="str">
         <f>IF('Filter Log'!B52="","",'Filter Log'!B52)</f>
         <v/>
       </c>
-      <c r="C52" s="20">
+      <c r="C52" s="20" t="str">
         <f>IF('Filter Log'!C52="","",'Filter Log'!C52)</f>
         <v/>
       </c>
-      <c r="D52" s="20">
+      <c r="D52" s="20" t="str">
         <f>IF('Filter Log'!D52="","",'Filter Log'!D52)</f>
         <v/>
       </c>
-      <c r="E52" s="20">
+      <c r="E52" s="20" t="str">
         <f>IF('Filter Log'!E52="","",'Filter Log'!E52)</f>
         <v/>
       </c>
@@ -3620,23 +3620,23 @@
       <c r="G52" s="22" t="n"/>
     </row>
     <row r="53" ht="26" customHeight="1">
-      <c r="A53" s="20">
+      <c r="A53" s="20" t="str">
         <f>IF('Filter Log'!A53="","",'Filter Log'!A53)</f>
         <v/>
       </c>
-      <c r="B53" s="21">
+      <c r="B53" s="21" t="str">
         <f>IF('Filter Log'!B53="","",'Filter Log'!B53)</f>
         <v/>
       </c>
-      <c r="C53" s="20">
+      <c r="C53" s="20" t="str">
         <f>IF('Filter Log'!C53="","",'Filter Log'!C53)</f>
         <v/>
       </c>
-      <c r="D53" s="20">
+      <c r="D53" s="20" t="str">
         <f>IF('Filter Log'!D53="","",'Filter Log'!D53)</f>
         <v/>
       </c>
-      <c r="E53" s="20">
+      <c r="E53" s="20" t="str">
         <f>IF('Filter Log'!E53="","",'Filter Log'!E53)</f>
         <v/>
       </c>
@@ -3644,23 +3644,23 @@
       <c r="G53" s="22" t="n"/>
     </row>
     <row r="54" ht="26" customHeight="1">
-      <c r="A54" s="20">
+      <c r="A54" s="20" t="str">
         <f>IF('Filter Log'!A54="","",'Filter Log'!A54)</f>
         <v/>
       </c>
-      <c r="B54" s="21">
+      <c r="B54" s="21" t="str">
         <f>IF('Filter Log'!B54="","",'Filter Log'!B54)</f>
         <v/>
       </c>
-      <c r="C54" s="20">
+      <c r="C54" s="20" t="str">
         <f>IF('Filter Log'!C54="","",'Filter Log'!C54)</f>
         <v/>
       </c>
-      <c r="D54" s="20">
+      <c r="D54" s="20" t="str">
         <f>IF('Filter Log'!D54="","",'Filter Log'!D54)</f>
         <v/>
       </c>
-      <c r="E54" s="20">
+      <c r="E54" s="20" t="str">
         <f>IF('Filter Log'!E54="","",'Filter Log'!E54)</f>
         <v/>
       </c>
@@ -3668,23 +3668,23 @@
       <c r="G54" s="22" t="n"/>
     </row>
     <row r="55" ht="26" customHeight="1">
-      <c r="A55" s="20">
+      <c r="A55" s="20" t="str">
         <f>IF('Filter Log'!A55="","",'Filter Log'!A55)</f>
         <v/>
       </c>
-      <c r="B55" s="21">
+      <c r="B55" s="21" t="str">
         <f>IF('Filter Log'!B55="","",'Filter Log'!B55)</f>
         <v/>
       </c>
-      <c r="C55" s="20">
+      <c r="C55" s="20" t="str">
         <f>IF('Filter Log'!C55="","",'Filter Log'!C55)</f>
         <v/>
       </c>
-      <c r="D55" s="20">
+      <c r="D55" s="20" t="str">
         <f>IF('Filter Log'!D55="","",'Filter Log'!D55)</f>
         <v/>
       </c>
-      <c r="E55" s="20">
+      <c r="E55" s="20" t="str">
         <f>IF('Filter Log'!E55="","",'Filter Log'!E55)</f>
         <v/>
       </c>
@@ -3692,23 +3692,23 @@
       <c r="G55" s="22" t="n"/>
     </row>
     <row r="56" ht="26" customHeight="1">
-      <c r="A56" s="20">
+      <c r="A56" s="20" t="str">
         <f>IF('Filter Log'!A56="","",'Filter Log'!A56)</f>
         <v/>
       </c>
-      <c r="B56" s="21">
+      <c r="B56" s="21" t="str">
         <f>IF('Filter Log'!B56="","",'Filter Log'!B56)</f>
         <v/>
       </c>
-      <c r="C56" s="20">
+      <c r="C56" s="20" t="str">
         <f>IF('Filter Log'!C56="","",'Filter Log'!C56)</f>
         <v/>
       </c>
-      <c r="D56" s="20">
+      <c r="D56" s="20" t="str">
         <f>IF('Filter Log'!D56="","",'Filter Log'!D56)</f>
         <v/>
       </c>
-      <c r="E56" s="20">
+      <c r="E56" s="20" t="str">
         <f>IF('Filter Log'!E56="","",'Filter Log'!E56)</f>
         <v/>
       </c>
@@ -3716,23 +3716,23 @@
       <c r="G56" s="22" t="n"/>
     </row>
     <row r="57" ht="26" customHeight="1">
-      <c r="A57" s="20">
+      <c r="A57" s="20" t="str">
         <f>IF('Filter Log'!A57="","",'Filter Log'!A57)</f>
         <v/>
       </c>
-      <c r="B57" s="21">
+      <c r="B57" s="21" t="str">
         <f>IF('Filter Log'!B57="","",'Filter Log'!B57)</f>
         <v/>
       </c>
-      <c r="C57" s="20">
+      <c r="C57" s="20" t="str">
         <f>IF('Filter Log'!C57="","",'Filter Log'!C57)</f>
         <v/>
       </c>
-      <c r="D57" s="20">
+      <c r="D57" s="20" t="str">
         <f>IF('Filter Log'!D57="","",'Filter Log'!D57)</f>
         <v/>
       </c>
-      <c r="E57" s="20">
+      <c r="E57" s="20" t="str">
         <f>IF('Filter Log'!E57="","",'Filter Log'!E57)</f>
         <v/>
       </c>
@@ -3740,23 +3740,23 @@
       <c r="G57" s="22" t="n"/>
     </row>
     <row r="58" ht="26" customHeight="1">
-      <c r="A58" s="20">
+      <c r="A58" s="20" t="str">
         <f>IF('Filter Log'!A58="","",'Filter Log'!A58)</f>
         <v/>
       </c>
-      <c r="B58" s="21">
+      <c r="B58" s="21" t="str">
         <f>IF('Filter Log'!B58="","",'Filter Log'!B58)</f>
         <v/>
       </c>
-      <c r="C58" s="20">
+      <c r="C58" s="20" t="str">
         <f>IF('Filter Log'!C58="","",'Filter Log'!C58)</f>
         <v/>
       </c>
-      <c r="D58" s="20">
+      <c r="D58" s="20" t="str">
         <f>IF('Filter Log'!D58="","",'Filter Log'!D58)</f>
         <v/>
       </c>
-      <c r="E58" s="20">
+      <c r="E58" s="20" t="str">
         <f>IF('Filter Log'!E58="","",'Filter Log'!E58)</f>
         <v/>
       </c>
@@ -3764,23 +3764,23 @@
       <c r="G58" s="22" t="n"/>
     </row>
     <row r="59" ht="26" customHeight="1">
-      <c r="A59" s="20">
+      <c r="A59" s="20" t="str">
         <f>IF('Filter Log'!A59="","",'Filter Log'!A59)</f>
         <v/>
       </c>
-      <c r="B59" s="21">
+      <c r="B59" s="21" t="str">
         <f>IF('Filter Log'!B59="","",'Filter Log'!B59)</f>
         <v/>
       </c>
-      <c r="C59" s="20">
+      <c r="C59" s="20" t="str">
         <f>IF('Filter Log'!C59="","",'Filter Log'!C59)</f>
         <v/>
       </c>
-      <c r="D59" s="20">
+      <c r="D59" s="20" t="str">
         <f>IF('Filter Log'!D59="","",'Filter Log'!D59)</f>
         <v/>
       </c>
-      <c r="E59" s="20">
+      <c r="E59" s="20" t="str">
         <f>IF('Filter Log'!E59="","",'Filter Log'!E59)</f>
         <v/>
       </c>
@@ -3788,23 +3788,23 @@
       <c r="G59" s="22" t="n"/>
     </row>
     <row r="60" ht="26" customHeight="1">
-      <c r="A60" s="20">
+      <c r="A60" s="20" t="str">
         <f>IF('Filter Log'!A60="","",'Filter Log'!A60)</f>
         <v/>
       </c>
-      <c r="B60" s="21">
+      <c r="B60" s="21" t="str">
         <f>IF('Filter Log'!B60="","",'Filter Log'!B60)</f>
         <v/>
       </c>
-      <c r="C60" s="20">
+      <c r="C60" s="20" t="str">
         <f>IF('Filter Log'!C60="","",'Filter Log'!C60)</f>
         <v/>
       </c>
-      <c r="D60" s="20">
+      <c r="D60" s="20" t="str">
         <f>IF('Filter Log'!D60="","",'Filter Log'!D60)</f>
         <v/>
       </c>
-      <c r="E60" s="20">
+      <c r="E60" s="20" t="str">
         <f>IF('Filter Log'!E60="","",'Filter Log'!E60)</f>
         <v/>
       </c>
@@ -3812,23 +3812,23 @@
       <c r="G60" s="22" t="n"/>
     </row>
     <row r="61" ht="26" customHeight="1">
-      <c r="A61" s="20">
+      <c r="A61" s="20" t="str">
         <f>IF('Filter Log'!A61="","",'Filter Log'!A61)</f>
         <v/>
       </c>
-      <c r="B61" s="21">
+      <c r="B61" s="21" t="str">
         <f>IF('Filter Log'!B61="","",'Filter Log'!B61)</f>
         <v/>
       </c>
-      <c r="C61" s="20">
+      <c r="C61" s="20" t="str">
         <f>IF('Filter Log'!C61="","",'Filter Log'!C61)</f>
         <v/>
       </c>
-      <c r="D61" s="20">
+      <c r="D61" s="20" t="str">
         <f>IF('Filter Log'!D61="","",'Filter Log'!D61)</f>
         <v/>
       </c>
-      <c r="E61" s="20">
+      <c r="E61" s="20" t="str">
         <f>IF('Filter Log'!E61="","",'Filter Log'!E61)</f>
         <v/>
       </c>
@@ -3836,23 +3836,23 @@
       <c r="G61" s="22" t="n"/>
     </row>
     <row r="62" ht="26" customHeight="1">
-      <c r="A62" s="20">
+      <c r="A62" s="20" t="str">
         <f>IF('Filter Log'!A62="","",'Filter Log'!A62)</f>
         <v/>
       </c>
-      <c r="B62" s="21">
+      <c r="B62" s="21" t="str">
         <f>IF('Filter Log'!B62="","",'Filter Log'!B62)</f>
         <v/>
       </c>
-      <c r="C62" s="20">
+      <c r="C62" s="20" t="str">
         <f>IF('Filter Log'!C62="","",'Filter Log'!C62)</f>
         <v/>
       </c>
-      <c r="D62" s="20">
+      <c r="D62" s="20" t="str">
         <f>IF('Filter Log'!D62="","",'Filter Log'!D62)</f>
         <v/>
       </c>
-      <c r="E62" s="20">
+      <c r="E62" s="20" t="str">
         <f>IF('Filter Log'!E62="","",'Filter Log'!E62)</f>
         <v/>
       </c>
@@ -3860,23 +3860,23 @@
       <c r="G62" s="22" t="n"/>
     </row>
     <row r="63" ht="26" customHeight="1">
-      <c r="A63" s="20">
+      <c r="A63" s="20" t="str">
         <f>IF('Filter Log'!A63="","",'Filter Log'!A63)</f>
         <v/>
       </c>
-      <c r="B63" s="21">
+      <c r="B63" s="21" t="str">
         <f>IF('Filter Log'!B63="","",'Filter Log'!B63)</f>
         <v/>
       </c>
-      <c r="C63" s="20">
+      <c r="C63" s="20" t="str">
         <f>IF('Filter Log'!C63="","",'Filter Log'!C63)</f>
         <v/>
       </c>
-      <c r="D63" s="20">
+      <c r="D63" s="20" t="str">
         <f>IF('Filter Log'!D63="","",'Filter Log'!D63)</f>
         <v/>
       </c>
-      <c r="E63" s="20">
+      <c r="E63" s="20" t="str">
         <f>IF('Filter Log'!E63="","",'Filter Log'!E63)</f>
         <v/>
       </c>
@@ -3884,23 +3884,23 @@
       <c r="G63" s="22" t="n"/>
     </row>
     <row r="64" ht="26" customHeight="1">
-      <c r="A64" s="20">
+      <c r="A64" s="20" t="str">
         <f>IF('Filter Log'!A64="","",'Filter Log'!A64)</f>
         <v/>
       </c>
-      <c r="B64" s="21">
+      <c r="B64" s="21" t="str">
         <f>IF('Filter Log'!B64="","",'Filter Log'!B64)</f>
         <v/>
       </c>
-      <c r="C64" s="20">
+      <c r="C64" s="20" t="str">
         <f>IF('Filter Log'!C64="","",'Filter Log'!C64)</f>
         <v/>
       </c>
-      <c r="D64" s="20">
+      <c r="D64" s="20" t="str">
         <f>IF('Filter Log'!D64="","",'Filter Log'!D64)</f>
         <v/>
       </c>
-      <c r="E64" s="20">
+      <c r="E64" s="20" t="str">
         <f>IF('Filter Log'!E64="","",'Filter Log'!E64)</f>
         <v/>
       </c>
@@ -3908,23 +3908,23 @@
       <c r="G64" s="22" t="n"/>
     </row>
     <row r="65" ht="26" customHeight="1">
-      <c r="A65" s="20">
+      <c r="A65" s="20" t="str">
         <f>IF('Filter Log'!A65="","",'Filter Log'!A65)</f>
         <v/>
       </c>
-      <c r="B65" s="21">
+      <c r="B65" s="21" t="str">
         <f>IF('Filter Log'!B65="","",'Filter Log'!B65)</f>
         <v/>
       </c>
-      <c r="C65" s="20">
+      <c r="C65" s="20" t="str">
         <f>IF('Filter Log'!C65="","",'Filter Log'!C65)</f>
         <v/>
       </c>
-      <c r="D65" s="20">
+      <c r="D65" s="20" t="str">
         <f>IF('Filter Log'!D65="","",'Filter Log'!D65)</f>
         <v/>
       </c>
-      <c r="E65" s="20">
+      <c r="E65" s="20" t="str">
         <f>IF('Filter Log'!E65="","",'Filter Log'!E65)</f>
         <v/>
       </c>
@@ -3932,23 +3932,23 @@
       <c r="G65" s="22" t="n"/>
     </row>
     <row r="66" ht="26" customHeight="1">
-      <c r="A66" s="20">
+      <c r="A66" s="20" t="str">
         <f>IF('Filter Log'!A66="","",'Filter Log'!A66)</f>
         <v/>
       </c>
-      <c r="B66" s="21">
+      <c r="B66" s="21" t="str">
         <f>IF('Filter Log'!B66="","",'Filter Log'!B66)</f>
         <v/>
       </c>
-      <c r="C66" s="20">
+      <c r="C66" s="20" t="str">
         <f>IF('Filter Log'!C66="","",'Filter Log'!C66)</f>
         <v/>
       </c>
-      <c r="D66" s="20">
+      <c r="D66" s="20" t="str">
         <f>IF('Filter Log'!D66="","",'Filter Log'!D66)</f>
         <v/>
       </c>
-      <c r="E66" s="20">
+      <c r="E66" s="20" t="str">
         <f>IF('Filter Log'!E66="","",'Filter Log'!E66)</f>
         <v/>
       </c>
@@ -3956,23 +3956,23 @@
       <c r="G66" s="22" t="n"/>
     </row>
     <row r="67" ht="26" customHeight="1">
-      <c r="A67" s="20">
+      <c r="A67" s="20" t="str">
         <f>IF('Filter Log'!A67="","",'Filter Log'!A67)</f>
         <v/>
       </c>
-      <c r="B67" s="21">
+      <c r="B67" s="21" t="str">
         <f>IF('Filter Log'!B67="","",'Filter Log'!B67)</f>
         <v/>
       </c>
-      <c r="C67" s="20">
+      <c r="C67" s="20" t="str">
         <f>IF('Filter Log'!C67="","",'Filter Log'!C67)</f>
         <v/>
       </c>
-      <c r="D67" s="20">
+      <c r="D67" s="20" t="str">
         <f>IF('Filter Log'!D67="","",'Filter Log'!D67)</f>
         <v/>
       </c>
-      <c r="E67" s="20">
+      <c r="E67" s="20" t="str">
         <f>IF('Filter Log'!E67="","",'Filter Log'!E67)</f>
         <v/>
       </c>
@@ -3980,23 +3980,23 @@
       <c r="G67" s="22" t="n"/>
     </row>
     <row r="68" ht="26" customHeight="1">
-      <c r="A68" s="20">
+      <c r="A68" s="20" t="str">
         <f>IF('Filter Log'!A68="","",'Filter Log'!A68)</f>
         <v/>
       </c>
-      <c r="B68" s="21">
+      <c r="B68" s="21" t="str">
         <f>IF('Filter Log'!B68="","",'Filter Log'!B68)</f>
         <v/>
       </c>
-      <c r="C68" s="20">
+      <c r="C68" s="20" t="str">
         <f>IF('Filter Log'!C68="","",'Filter Log'!C68)</f>
         <v/>
       </c>
-      <c r="D68" s="20">
+      <c r="D68" s="20" t="str">
         <f>IF('Filter Log'!D68="","",'Filter Log'!D68)</f>
         <v/>
       </c>
-      <c r="E68" s="20">
+      <c r="E68" s="20" t="str">
         <f>IF('Filter Log'!E68="","",'Filter Log'!E68)</f>
         <v/>
       </c>
@@ -4004,23 +4004,23 @@
       <c r="G68" s="22" t="n"/>
     </row>
     <row r="69" ht="26" customHeight="1">
-      <c r="A69" s="20">
+      <c r="A69" s="20" t="str">
         <f>IF('Filter Log'!A69="","",'Filter Log'!A69)</f>
         <v/>
       </c>
-      <c r="B69" s="21">
+      <c r="B69" s="21" t="str">
         <f>IF('Filter Log'!B69="","",'Filter Log'!B69)</f>
         <v/>
       </c>
-      <c r="C69" s="20">
+      <c r="C69" s="20" t="str">
         <f>IF('Filter Log'!C69="","",'Filter Log'!C69)</f>
         <v/>
       </c>
-      <c r="D69" s="20">
+      <c r="D69" s="20" t="str">
         <f>IF('Filter Log'!D69="","",'Filter Log'!D69)</f>
         <v/>
       </c>
-      <c r="E69" s="20">
+      <c r="E69" s="20" t="str">
         <f>IF('Filter Log'!E69="","",'Filter Log'!E69)</f>
         <v/>
       </c>
@@ -4028,23 +4028,23 @@
       <c r="G69" s="22" t="n"/>
     </row>
     <row r="70" ht="26" customHeight="1">
-      <c r="A70" s="20">
+      <c r="A70" s="20" t="str">
         <f>IF('Filter Log'!A70="","",'Filter Log'!A70)</f>
         <v/>
       </c>
-      <c r="B70" s="21">
+      <c r="B70" s="21" t="str">
         <f>IF('Filter Log'!B70="","",'Filter Log'!B70)</f>
         <v/>
       </c>
-      <c r="C70" s="20">
+      <c r="C70" s="20" t="str">
         <f>IF('Filter Log'!C70="","",'Filter Log'!C70)</f>
         <v/>
       </c>
-      <c r="D70" s="20">
+      <c r="D70" s="20" t="str">
         <f>IF('Filter Log'!D70="","",'Filter Log'!D70)</f>
         <v/>
       </c>
-      <c r="E70" s="20">
+      <c r="E70" s="20" t="str">
         <f>IF('Filter Log'!E70="","",'Filter Log'!E70)</f>
         <v/>
       </c>
@@ -4052,23 +4052,23 @@
       <c r="G70" s="22" t="n"/>
     </row>
     <row r="71" ht="26" customHeight="1">
-      <c r="A71" s="20">
+      <c r="A71" s="20" t="str">
         <f>IF('Filter Log'!A71="","",'Filter Log'!A71)</f>
         <v/>
       </c>
-      <c r="B71" s="21">
+      <c r="B71" s="21" t="str">
         <f>IF('Filter Log'!B71="","",'Filter Log'!B71)</f>
         <v/>
       </c>
-      <c r="C71" s="20">
+      <c r="C71" s="20" t="str">
         <f>IF('Filter Log'!C71="","",'Filter Log'!C71)</f>
         <v/>
       </c>
-      <c r="D71" s="20">
+      <c r="D71" s="20" t="str">
         <f>IF('Filter Log'!D71="","",'Filter Log'!D71)</f>
         <v/>
       </c>
-      <c r="E71" s="20">
+      <c r="E71" s="20" t="str">
         <f>IF('Filter Log'!E71="","",'Filter Log'!E71)</f>
         <v/>
       </c>
@@ -4076,23 +4076,23 @@
       <c r="G71" s="22" t="n"/>
     </row>
     <row r="72" ht="26" customHeight="1">
-      <c r="A72" s="20">
+      <c r="A72" s="20" t="str">
         <f>IF('Filter Log'!A72="","",'Filter Log'!A72)</f>
         <v/>
       </c>
-      <c r="B72" s="21">
+      <c r="B72" s="21" t="str">
         <f>IF('Filter Log'!B72="","",'Filter Log'!B72)</f>
         <v/>
       </c>
-      <c r="C72" s="20">
+      <c r="C72" s="20" t="str">
         <f>IF('Filter Log'!C72="","",'Filter Log'!C72)</f>
         <v/>
       </c>
-      <c r="D72" s="20">
+      <c r="D72" s="20" t="str">
         <f>IF('Filter Log'!D72="","",'Filter Log'!D72)</f>
         <v/>
       </c>
-      <c r="E72" s="20">
+      <c r="E72" s="20" t="str">
         <f>IF('Filter Log'!E72="","",'Filter Log'!E72)</f>
         <v/>
       </c>
@@ -4100,23 +4100,23 @@
       <c r="G72" s="22" t="n"/>
     </row>
     <row r="73" ht="26" customHeight="1">
-      <c r="A73" s="20">
+      <c r="A73" s="20" t="str">
         <f>IF('Filter Log'!A73="","",'Filter Log'!A73)</f>
         <v/>
       </c>
-      <c r="B73" s="21">
+      <c r="B73" s="21" t="str">
         <f>IF('Filter Log'!B73="","",'Filter Log'!B73)</f>
         <v/>
       </c>
-      <c r="C73" s="20">
+      <c r="C73" s="20" t="str">
         <f>IF('Filter Log'!C73="","",'Filter Log'!C73)</f>
         <v/>
       </c>
-      <c r="D73" s="20">
+      <c r="D73" s="20" t="str">
         <f>IF('Filter Log'!D73="","",'Filter Log'!D73)</f>
         <v/>
       </c>
-      <c r="E73" s="20">
+      <c r="E73" s="20" t="str">
         <f>IF('Filter Log'!E73="","",'Filter Log'!E73)</f>
         <v/>
       </c>
@@ -4124,23 +4124,23 @@
       <c r="G73" s="22" t="n"/>
     </row>
     <row r="74" ht="26" customHeight="1">
-      <c r="A74" s="20">
+      <c r="A74" s="20" t="str">
         <f>IF('Filter Log'!A74="","",'Filter Log'!A74)</f>
         <v/>
       </c>
-      <c r="B74" s="21">
+      <c r="B74" s="21" t="str">
         <f>IF('Filter Log'!B74="","",'Filter Log'!B74)</f>
         <v/>
       </c>
-      <c r="C74" s="20">
+      <c r="C74" s="20" t="str">
         <f>IF('Filter Log'!C74="","",'Filter Log'!C74)</f>
         <v/>
       </c>
-      <c r="D74" s="20">
+      <c r="D74" s="20" t="str">
         <f>IF('Filter Log'!D74="","",'Filter Log'!D74)</f>
         <v/>
       </c>
-      <c r="E74" s="20">
+      <c r="E74" s="20" t="str">
         <f>IF('Filter Log'!E74="","",'Filter Log'!E74)</f>
         <v/>
       </c>
@@ -4148,23 +4148,23 @@
       <c r="G74" s="22" t="n"/>
     </row>
     <row r="75" ht="26" customHeight="1">
-      <c r="A75" s="20">
+      <c r="A75" s="20" t="str">
         <f>IF('Filter Log'!A75="","",'Filter Log'!A75)</f>
         <v/>
       </c>
-      <c r="B75" s="21">
+      <c r="B75" s="21" t="str">
         <f>IF('Filter Log'!B75="","",'Filter Log'!B75)</f>
         <v/>
       </c>
-      <c r="C75" s="20">
+      <c r="C75" s="20" t="str">
         <f>IF('Filter Log'!C75="","",'Filter Log'!C75)</f>
         <v/>
       </c>
-      <c r="D75" s="20">
+      <c r="D75" s="20" t="str">
         <f>IF('Filter Log'!D75="","",'Filter Log'!D75)</f>
         <v/>
       </c>
-      <c r="E75" s="20">
+      <c r="E75" s="20" t="str">
         <f>IF('Filter Log'!E75="","",'Filter Log'!E75)</f>
         <v/>
       </c>
@@ -4172,23 +4172,23 @@
       <c r="G75" s="22" t="n"/>
     </row>
     <row r="76" ht="26" customHeight="1">
-      <c r="A76" s="20">
+      <c r="A76" s="20" t="str">
         <f>IF('Filter Log'!A76="","",'Filter Log'!A76)</f>
         <v/>
       </c>
-      <c r="B76" s="21">
+      <c r="B76" s="21" t="str">
         <f>IF('Filter Log'!B76="","",'Filter Log'!B76)</f>
         <v/>
       </c>
-      <c r="C76" s="20">
+      <c r="C76" s="20" t="str">
         <f>IF('Filter Log'!C76="","",'Filter Log'!C76)</f>
         <v/>
       </c>
-      <c r="D76" s="20">
+      <c r="D76" s="20" t="str">
         <f>IF('Filter Log'!D76="","",'Filter Log'!D76)</f>
         <v/>
       </c>
-      <c r="E76" s="20">
+      <c r="E76" s="20" t="str">
         <f>IF('Filter Log'!E76="","",'Filter Log'!E76)</f>
         <v/>
       </c>
@@ -4196,23 +4196,23 @@
       <c r="G76" s="22" t="n"/>
     </row>
     <row r="77" ht="26" customHeight="1">
-      <c r="A77" s="20">
+      <c r="A77" s="20" t="str">
         <f>IF('Filter Log'!A77="","",'Filter Log'!A77)</f>
         <v/>
       </c>
-      <c r="B77" s="21">
+      <c r="B77" s="21" t="str">
         <f>IF('Filter Log'!B77="","",'Filter Log'!B77)</f>
         <v/>
       </c>
-      <c r="C77" s="20">
+      <c r="C77" s="20" t="str">
         <f>IF('Filter Log'!C77="","",'Filter Log'!C77)</f>
         <v/>
       </c>
-      <c r="D77" s="20">
+      <c r="D77" s="20" t="str">
         <f>IF('Filter Log'!D77="","",'Filter Log'!D77)</f>
         <v/>
       </c>
-      <c r="E77" s="20">
+      <c r="E77" s="20" t="str">
         <f>IF('Filter Log'!E77="","",'Filter Log'!E77)</f>
         <v/>
       </c>
@@ -4220,23 +4220,23 @@
       <c r="G77" s="22" t="n"/>
     </row>
     <row r="78" ht="26" customHeight="1">
-      <c r="A78" s="20">
+      <c r="A78" s="20" t="str">
         <f>IF('Filter Log'!A78="","",'Filter Log'!A78)</f>
         <v/>
       </c>
-      <c r="B78" s="21">
+      <c r="B78" s="21" t="str">
         <f>IF('Filter Log'!B78="","",'Filter Log'!B78)</f>
         <v/>
       </c>
-      <c r="C78" s="20">
+      <c r="C78" s="20" t="str">
         <f>IF('Filter Log'!C78="","",'Filter Log'!C78)</f>
         <v/>
       </c>
-      <c r="D78" s="20">
+      <c r="D78" s="20" t="str">
         <f>IF('Filter Log'!D78="","",'Filter Log'!D78)</f>
         <v/>
       </c>
-      <c r="E78" s="20">
+      <c r="E78" s="20" t="str">
         <f>IF('Filter Log'!E78="","",'Filter Log'!E78)</f>
         <v/>
       </c>
@@ -4244,23 +4244,23 @@
       <c r="G78" s="22" t="n"/>
     </row>
     <row r="79" ht="26" customHeight="1">
-      <c r="A79" s="20">
+      <c r="A79" s="20" t="str">
         <f>IF('Filter Log'!A79="","",'Filter Log'!A79)</f>
         <v/>
       </c>
-      <c r="B79" s="21">
+      <c r="B79" s="21" t="str">
         <f>IF('Filter Log'!B79="","",'Filter Log'!B79)</f>
         <v/>
       </c>
-      <c r="C79" s="20">
+      <c r="C79" s="20" t="str">
         <f>IF('Filter Log'!C79="","",'Filter Log'!C79)</f>
         <v/>
       </c>
-      <c r="D79" s="20">
+      <c r="D79" s="20" t="str">
         <f>IF('Filter Log'!D79="","",'Filter Log'!D79)</f>
         <v/>
       </c>
-      <c r="E79" s="20">
+      <c r="E79" s="20" t="str">
         <f>IF('Filter Log'!E79="","",'Filter Log'!E79)</f>
         <v/>
       </c>
@@ -4268,23 +4268,23 @@
       <c r="G79" s="22" t="n"/>
     </row>
     <row r="80" ht="26" customHeight="1">
-      <c r="A80" s="20">
+      <c r="A80" s="20" t="str">
         <f>IF('Filter Log'!A80="","",'Filter Log'!A80)</f>
         <v/>
       </c>
-      <c r="B80" s="21">
+      <c r="B80" s="21" t="str">
         <f>IF('Filter Log'!B80="","",'Filter Log'!B80)</f>
         <v/>
       </c>
-      <c r="C80" s="20">
+      <c r="C80" s="20" t="str">
         <f>IF('Filter Log'!C80="","",'Filter Log'!C80)</f>
         <v/>
       </c>
-      <c r="D80" s="20">
+      <c r="D80" s="20" t="str">
         <f>IF('Filter Log'!D80="","",'Filter Log'!D80)</f>
         <v/>
       </c>
-      <c r="E80" s="20">
+      <c r="E80" s="20" t="str">
         <f>IF('Filter Log'!E80="","",'Filter Log'!E80)</f>
         <v/>
       </c>
@@ -4292,23 +4292,23 @@
       <c r="G80" s="22" t="n"/>
     </row>
     <row r="81" ht="26" customHeight="1">
-      <c r="A81" s="20">
+      <c r="A81" s="20" t="str">
         <f>IF('Filter Log'!A81="","",'Filter Log'!A81)</f>
         <v/>
       </c>
-      <c r="B81" s="21">
+      <c r="B81" s="21" t="str">
         <f>IF('Filter Log'!B81="","",'Filter Log'!B81)</f>
         <v/>
       </c>
-      <c r="C81" s="20">
+      <c r="C81" s="20" t="str">
         <f>IF('Filter Log'!C81="","",'Filter Log'!C81)</f>
         <v/>
       </c>
-      <c r="D81" s="20">
+      <c r="D81" s="20" t="str">
         <f>IF('Filter Log'!D81="","",'Filter Log'!D81)</f>
         <v/>
       </c>
-      <c r="E81" s="20">
+      <c r="E81" s="20" t="str">
         <f>IF('Filter Log'!E81="","",'Filter Log'!E81)</f>
         <v/>
       </c>
@@ -4316,23 +4316,23 @@
       <c r="G81" s="22" t="n"/>
     </row>
     <row r="82" ht="26" customHeight="1">
-      <c r="A82" s="20">
+      <c r="A82" s="20" t="str">
         <f>IF('Filter Log'!A82="","",'Filter Log'!A82)</f>
         <v/>
       </c>
-      <c r="B82" s="21">
+      <c r="B82" s="21" t="str">
         <f>IF('Filter Log'!B82="","",'Filter Log'!B82)</f>
         <v/>
       </c>
-      <c r="C82" s="20">
+      <c r="C82" s="20" t="str">
         <f>IF('Filter Log'!C82="","",'Filter Log'!C82)</f>
         <v/>
       </c>
-      <c r="D82" s="20">
+      <c r="D82" s="20" t="str">
         <f>IF('Filter Log'!D82="","",'Filter Log'!D82)</f>
         <v/>
       </c>
-      <c r="E82" s="20">
+      <c r="E82" s="20" t="str">
         <f>IF('Filter Log'!E82="","",'Filter Log'!E82)</f>
         <v/>
       </c>
@@ -4340,23 +4340,23 @@
       <c r="G82" s="22" t="n"/>
     </row>
     <row r="83" ht="26" customHeight="1">
-      <c r="A83" s="20">
+      <c r="A83" s="20" t="str">
         <f>IF('Filter Log'!A83="","",'Filter Log'!A83)</f>
         <v/>
       </c>
-      <c r="B83" s="21">
+      <c r="B83" s="21" t="str">
         <f>IF('Filter Log'!B83="","",'Filter Log'!B83)</f>
         <v/>
       </c>
-      <c r="C83" s="20">
+      <c r="C83" s="20" t="str">
         <f>IF('Filter Log'!C83="","",'Filter Log'!C83)</f>
         <v/>
       </c>
-      <c r="D83" s="20">
+      <c r="D83" s="20" t="str">
         <f>IF('Filter Log'!D83="","",'Filter Log'!D83)</f>
         <v/>
       </c>
-      <c r="E83" s="20">
+      <c r="E83" s="20" t="str">
         <f>IF('Filter Log'!E83="","",'Filter Log'!E83)</f>
         <v/>
       </c>
@@ -4364,23 +4364,23 @@
       <c r="G83" s="22" t="n"/>
     </row>
     <row r="84" ht="26" customHeight="1">
-      <c r="A84" s="20">
+      <c r="A84" s="20" t="str">
         <f>IF('Filter Log'!A84="","",'Filter Log'!A84)</f>
         <v/>
       </c>
-      <c r="B84" s="21">
+      <c r="B84" s="21" t="str">
         <f>IF('Filter Log'!B84="","",'Filter Log'!B84)</f>
         <v/>
       </c>
-      <c r="C84" s="20">
+      <c r="C84" s="20" t="str">
         <f>IF('Filter Log'!C84="","",'Filter Log'!C84)</f>
         <v/>
       </c>
-      <c r="D84" s="20">
+      <c r="D84" s="20" t="str">
         <f>IF('Filter Log'!D84="","",'Filter Log'!D84)</f>
         <v/>
       </c>
-      <c r="E84" s="20">
+      <c r="E84" s="20" t="str">
         <f>IF('Filter Log'!E84="","",'Filter Log'!E84)</f>
         <v/>
       </c>
@@ -4388,23 +4388,23 @@
       <c r="G84" s="22" t="n"/>
     </row>
     <row r="85" ht="26" customHeight="1">
-      <c r="A85" s="20">
+      <c r="A85" s="20" t="str">
         <f>IF('Filter Log'!A85="","",'Filter Log'!A85)</f>
         <v/>
       </c>
-      <c r="B85" s="21">
+      <c r="B85" s="21" t="str">
         <f>IF('Filter Log'!B85="","",'Filter Log'!B85)</f>
         <v/>
       </c>
-      <c r="C85" s="20">
+      <c r="C85" s="20" t="str">
         <f>IF('Filter Log'!C85="","",'Filter Log'!C85)</f>
         <v/>
       </c>
-      <c r="D85" s="20">
+      <c r="D85" s="20" t="str">
         <f>IF('Filter Log'!D85="","",'Filter Log'!D85)</f>
         <v/>
       </c>
-      <c r="E85" s="20">
+      <c r="E85" s="20" t="str">
         <f>IF('Filter Log'!E85="","",'Filter Log'!E85)</f>
         <v/>
       </c>
@@ -4412,23 +4412,23 @@
       <c r="G85" s="22" t="n"/>
     </row>
     <row r="86" ht="26" customHeight="1">
-      <c r="A86" s="20">
+      <c r="A86" s="20" t="str">
         <f>IF('Filter Log'!A86="","",'Filter Log'!A86)</f>
         <v/>
       </c>
-      <c r="B86" s="21">
+      <c r="B86" s="21" t="str">
         <f>IF('Filter Log'!B86="","",'Filter Log'!B86)</f>
         <v/>
       </c>
-      <c r="C86" s="20">
+      <c r="C86" s="20" t="str">
         <f>IF('Filter Log'!C86="","",'Filter Log'!C86)</f>
         <v/>
       </c>
-      <c r="D86" s="20">
+      <c r="D86" s="20" t="str">
         <f>IF('Filter Log'!D86="","",'Filter Log'!D86)</f>
         <v/>
       </c>
-      <c r="E86" s="20">
+      <c r="E86" s="20" t="str">
         <f>IF('Filter Log'!E86="","",'Filter Log'!E86)</f>
         <v/>
       </c>
@@ -4436,23 +4436,23 @@
       <c r="G86" s="22" t="n"/>
     </row>
     <row r="87" ht="26" customHeight="1">
-      <c r="A87" s="20">
+      <c r="A87" s="20" t="str">
         <f>IF('Filter Log'!A87="","",'Filter Log'!A87)</f>
         <v/>
       </c>
-      <c r="B87" s="21">
+      <c r="B87" s="21" t="str">
         <f>IF('Filter Log'!B87="","",'Filter Log'!B87)</f>
         <v/>
       </c>
-      <c r="C87" s="20">
+      <c r="C87" s="20" t="str">
         <f>IF('Filter Log'!C87="","",'Filter Log'!C87)</f>
         <v/>
       </c>
-      <c r="D87" s="20">
+      <c r="D87" s="20" t="str">
         <f>IF('Filter Log'!D87="","",'Filter Log'!D87)</f>
         <v/>
       </c>
-      <c r="E87" s="20">
+      <c r="E87" s="20" t="str">
         <f>IF('Filter Log'!E87="","",'Filter Log'!E87)</f>
         <v/>
       </c>
@@ -4460,23 +4460,23 @@
       <c r="G87" s="22" t="n"/>
     </row>
     <row r="88" ht="26" customHeight="1">
-      <c r="A88" s="20">
+      <c r="A88" s="20" t="str">
         <f>IF('Filter Log'!A88="","",'Filter Log'!A88)</f>
         <v/>
       </c>
-      <c r="B88" s="21">
+      <c r="B88" s="21" t="str">
         <f>IF('Filter Log'!B88="","",'Filter Log'!B88)</f>
         <v/>
       </c>
-      <c r="C88" s="20">
+      <c r="C88" s="20" t="str">
         <f>IF('Filter Log'!C88="","",'Filter Log'!C88)</f>
         <v/>
       </c>
-      <c r="D88" s="20">
+      <c r="D88" s="20" t="str">
         <f>IF('Filter Log'!D88="","",'Filter Log'!D88)</f>
         <v/>
       </c>
-      <c r="E88" s="20">
+      <c r="E88" s="20" t="str">
         <f>IF('Filter Log'!E88="","",'Filter Log'!E88)</f>
         <v/>
       </c>
@@ -4484,23 +4484,23 @@
       <c r="G88" s="22" t="n"/>
     </row>
     <row r="89" ht="26" customHeight="1">
-      <c r="A89" s="20">
+      <c r="A89" s="20" t="str">
         <f>IF('Filter Log'!A89="","",'Filter Log'!A89)</f>
         <v/>
       </c>
-      <c r="B89" s="21">
+      <c r="B89" s="21" t="str">
         <f>IF('Filter Log'!B89="","",'Filter Log'!B89)</f>
         <v/>
       </c>
-      <c r="C89" s="20">
+      <c r="C89" s="20" t="str">
         <f>IF('Filter Log'!C89="","",'Filter Log'!C89)</f>
         <v/>
       </c>
-      <c r="D89" s="20">
+      <c r="D89" s="20" t="str">
         <f>IF('Filter Log'!D89="","",'Filter Log'!D89)</f>
         <v/>
       </c>
-      <c r="E89" s="20">
+      <c r="E89" s="20" t="str">
         <f>IF('Filter Log'!E89="","",'Filter Log'!E89)</f>
         <v/>
       </c>
@@ -4508,23 +4508,23 @@
       <c r="G89" s="22" t="n"/>
     </row>
     <row r="90" ht="26" customHeight="1">
-      <c r="A90" s="20">
+      <c r="A90" s="20" t="str">
         <f>IF('Filter Log'!A90="","",'Filter Log'!A90)</f>
         <v/>
       </c>
-      <c r="B90" s="21">
+      <c r="B90" s="21" t="str">
         <f>IF('Filter Log'!B90="","",'Filter Log'!B90)</f>
         <v/>
       </c>
-      <c r="C90" s="20">
+      <c r="C90" s="20" t="str">
         <f>IF('Filter Log'!C90="","",'Filter Log'!C90)</f>
         <v/>
       </c>
-      <c r="D90" s="20">
+      <c r="D90" s="20" t="str">
         <f>IF('Filter Log'!D90="","",'Filter Log'!D90)</f>
         <v/>
       </c>
-      <c r="E90" s="20">
+      <c r="E90" s="20" t="str">
         <f>IF('Filter Log'!E90="","",'Filter Log'!E90)</f>
         <v/>
       </c>
@@ -4532,23 +4532,23 @@
       <c r="G90" s="22" t="n"/>
     </row>
     <row r="91" ht="26" customHeight="1">
-      <c r="A91" s="20">
+      <c r="A91" s="20" t="str">
         <f>IF('Filter Log'!A91="","",'Filter Log'!A91)</f>
         <v/>
       </c>
-      <c r="B91" s="21">
+      <c r="B91" s="21" t="str">
         <f>IF('Filter Log'!B91="","",'Filter Log'!B91)</f>
         <v/>
       </c>
-      <c r="C91" s="20">
+      <c r="C91" s="20" t="str">
         <f>IF('Filter Log'!C91="","",'Filter Log'!C91)</f>
         <v/>
       </c>
-      <c r="D91" s="20">
+      <c r="D91" s="20" t="str">
         <f>IF('Filter Log'!D91="","",'Filter Log'!D91)</f>
         <v/>
       </c>
-      <c r="E91" s="20">
+      <c r="E91" s="20" t="str">
         <f>IF('Filter Log'!E91="","",'Filter Log'!E91)</f>
         <v/>
       </c>
@@ -4556,23 +4556,23 @@
       <c r="G91" s="22" t="n"/>
     </row>
     <row r="92" ht="26" customHeight="1">
-      <c r="A92" s="20">
+      <c r="A92" s="20" t="str">
         <f>IF('Filter Log'!A92="","",'Filter Log'!A92)</f>
         <v/>
       </c>
-      <c r="B92" s="21">
+      <c r="B92" s="21" t="str">
         <f>IF('Filter Log'!B92="","",'Filter Log'!B92)</f>
         <v/>
       </c>
-      <c r="C92" s="20">
+      <c r="C92" s="20" t="str">
         <f>IF('Filter Log'!C92="","",'Filter Log'!C92)</f>
         <v/>
       </c>
-      <c r="D92" s="20">
+      <c r="D92" s="20" t="str">
         <f>IF('Filter Log'!D92="","",'Filter Log'!D92)</f>
         <v/>
       </c>
-      <c r="E92" s="20">
+      <c r="E92" s="20" t="str">
         <f>IF('Filter Log'!E92="","",'Filter Log'!E92)</f>
         <v/>
       </c>
@@ -4580,23 +4580,23 @@
       <c r="G92" s="22" t="n"/>
     </row>
     <row r="93" ht="26" customHeight="1">
-      <c r="A93" s="20">
+      <c r="A93" s="20" t="str">
         <f>IF('Filter Log'!A93="","",'Filter Log'!A93)</f>
         <v/>
       </c>
-      <c r="B93" s="21">
+      <c r="B93" s="21" t="str">
         <f>IF('Filter Log'!B93="","",'Filter Log'!B93)</f>
         <v/>
       </c>
-      <c r="C93" s="20">
+      <c r="C93" s="20" t="str">
         <f>IF('Filter Log'!C93="","",'Filter Log'!C93)</f>
         <v/>
       </c>
-      <c r="D93" s="20">
+      <c r="D93" s="20" t="str">
         <f>IF('Filter Log'!D93="","",'Filter Log'!D93)</f>
         <v/>
       </c>
-      <c r="E93" s="20">
+      <c r="E93" s="20" t="str">
         <f>IF('Filter Log'!E93="","",'Filter Log'!E93)</f>
         <v/>
       </c>
@@ -4604,23 +4604,23 @@
       <c r="G93" s="22" t="n"/>
     </row>
     <row r="94" ht="26" customHeight="1">
-      <c r="A94" s="20">
+      <c r="A94" s="20" t="str">
         <f>IF('Filter Log'!A94="","",'Filter Log'!A94)</f>
         <v/>
       </c>
-      <c r="B94" s="21">
+      <c r="B94" s="21" t="str">
         <f>IF('Filter Log'!B94="","",'Filter Log'!B94)</f>
         <v/>
       </c>
-      <c r="C94" s="20">
+      <c r="C94" s="20" t="str">
         <f>IF('Filter Log'!C94="","",'Filter Log'!C94)</f>
         <v/>
       </c>
-      <c r="D94" s="20">
+      <c r="D94" s="20" t="str">
         <f>IF('Filter Log'!D94="","",'Filter Log'!D94)</f>
         <v/>
       </c>
-      <c r="E94" s="20">
+      <c r="E94" s="20" t="str">
         <f>IF('Filter Log'!E94="","",'Filter Log'!E94)</f>
         <v/>
       </c>
@@ -4628,23 +4628,23 @@
       <c r="G94" s="22" t="n"/>
     </row>
     <row r="95" ht="26" customHeight="1">
-      <c r="A95" s="20">
+      <c r="A95" s="20" t="str">
         <f>IF('Filter Log'!A95="","",'Filter Log'!A95)</f>
         <v/>
       </c>
-      <c r="B95" s="21">
+      <c r="B95" s="21" t="str">
         <f>IF('Filter Log'!B95="","",'Filter Log'!B95)</f>
         <v/>
       </c>
-      <c r="C95" s="20">
+      <c r="C95" s="20" t="str">
         <f>IF('Filter Log'!C95="","",'Filter Log'!C95)</f>
         <v/>
       </c>
-      <c r="D95" s="20">
+      <c r="D95" s="20" t="str">
         <f>IF('Filter Log'!D95="","",'Filter Log'!D95)</f>
         <v/>
       </c>
-      <c r="E95" s="20">
+      <c r="E95" s="20" t="str">
         <f>IF('Filter Log'!E95="","",'Filter Log'!E95)</f>
         <v/>
       </c>
@@ -4652,23 +4652,23 @@
       <c r="G95" s="22" t="n"/>
     </row>
     <row r="96" ht="26" customHeight="1">
-      <c r="A96" s="20">
+      <c r="A96" s="20" t="str">
         <f>IF('Filter Log'!A96="","",'Filter Log'!A96)</f>
         <v/>
       </c>
-      <c r="B96" s="21">
+      <c r="B96" s="21" t="str">
         <f>IF('Filter Log'!B96="","",'Filter Log'!B96)</f>
         <v/>
       </c>
-      <c r="C96" s="20">
+      <c r="C96" s="20" t="str">
         <f>IF('Filter Log'!C96="","",'Filter Log'!C96)</f>
         <v/>
       </c>
-      <c r="D96" s="20">
+      <c r="D96" s="20" t="str">
         <f>IF('Filter Log'!D96="","",'Filter Log'!D96)</f>
         <v/>
       </c>
-      <c r="E96" s="20">
+      <c r="E96" s="20" t="str">
         <f>IF('Filter Log'!E96="","",'Filter Log'!E96)</f>
         <v/>
       </c>
@@ -4676,23 +4676,23 @@
       <c r="G96" s="22" t="n"/>
     </row>
     <row r="97" ht="26" customHeight="1">
-      <c r="A97" s="20">
+      <c r="A97" s="20" t="str">
         <f>IF('Filter Log'!A97="","",'Filter Log'!A97)</f>
         <v/>
       </c>
-      <c r="B97" s="21">
+      <c r="B97" s="21" t="str">
         <f>IF('Filter Log'!B97="","",'Filter Log'!B97)</f>
         <v/>
       </c>
-      <c r="C97" s="20">
+      <c r="C97" s="20" t="str">
         <f>IF('Filter Log'!C97="","",'Filter Log'!C97)</f>
         <v/>
       </c>
-      <c r="D97" s="20">
+      <c r="D97" s="20" t="str">
         <f>IF('Filter Log'!D97="","",'Filter Log'!D97)</f>
         <v/>
       </c>
-      <c r="E97" s="20">
+      <c r="E97" s="20" t="str">
         <f>IF('Filter Log'!E97="","",'Filter Log'!E97)</f>
         <v/>
       </c>
@@ -4700,23 +4700,23 @@
       <c r="G97" s="22" t="n"/>
     </row>
     <row r="98" ht="26" customHeight="1">
-      <c r="A98" s="20">
+      <c r="A98" s="20" t="str">
         <f>IF('Filter Log'!A98="","",'Filter Log'!A98)</f>
         <v/>
       </c>
-      <c r="B98" s="21">
+      <c r="B98" s="21" t="str">
         <f>IF('Filter Log'!B98="","",'Filter Log'!B98)</f>
         <v/>
       </c>
-      <c r="C98" s="20">
+      <c r="C98" s="20" t="str">
         <f>IF('Filter Log'!C98="","",'Filter Log'!C98)</f>
         <v/>
       </c>
-      <c r="D98" s="20">
+      <c r="D98" s="20" t="str">
         <f>IF('Filter Log'!D98="","",'Filter Log'!D98)</f>
         <v/>
       </c>
-      <c r="E98" s="20">
+      <c r="E98" s="20" t="str">
         <f>IF('Filter Log'!E98="","",'Filter Log'!E98)</f>
         <v/>
       </c>
@@ -4724,23 +4724,23 @@
       <c r="G98" s="22" t="n"/>
     </row>
     <row r="99" ht="26" customHeight="1">
-      <c r="A99" s="20">
+      <c r="A99" s="20" t="str">
         <f>IF('Filter Log'!A99="","",'Filter Log'!A99)</f>
         <v/>
       </c>
-      <c r="B99" s="21">
+      <c r="B99" s="21" t="str">
         <f>IF('Filter Log'!B99="","",'Filter Log'!B99)</f>
         <v/>
       </c>
-      <c r="C99" s="20">
+      <c r="C99" s="20" t="str">
         <f>IF('Filter Log'!C99="","",'Filter Log'!C99)</f>
         <v/>
       </c>
-      <c r="D99" s="20">
+      <c r="D99" s="20" t="str">
         <f>IF('Filter Log'!D99="","",'Filter Log'!D99)</f>
         <v/>
       </c>
-      <c r="E99" s="20">
+      <c r="E99" s="20" t="str">
         <f>IF('Filter Log'!E99="","",'Filter Log'!E99)</f>
         <v/>
       </c>
@@ -4748,23 +4748,23 @@
       <c r="G99" s="22" t="n"/>
     </row>
     <row r="100" ht="26" customHeight="1">
-      <c r="A100" s="20">
+      <c r="A100" s="20" t="str">
         <f>IF('Filter Log'!A100="","",'Filter Log'!A100)</f>
         <v/>
       </c>
-      <c r="B100" s="21">
+      <c r="B100" s="21" t="str">
         <f>IF('Filter Log'!B100="","",'Filter Log'!B100)</f>
         <v/>
       </c>
-      <c r="C100" s="20">
+      <c r="C100" s="20" t="str">
         <f>IF('Filter Log'!C100="","",'Filter Log'!C100)</f>
         <v/>
       </c>
-      <c r="D100" s="20">
+      <c r="D100" s="20" t="str">
         <f>IF('Filter Log'!D100="","",'Filter Log'!D100)</f>
         <v/>
       </c>
-      <c r="E100" s="20">
+      <c r="E100" s="20" t="str">
         <f>IF('Filter Log'!E100="","",'Filter Log'!E100)</f>
         <v/>
       </c>
@@ -4772,23 +4772,23 @@
       <c r="G100" s="22" t="n"/>
     </row>
     <row r="101" ht="26" customHeight="1">
-      <c r="A101" s="20">
+      <c r="A101" s="20" t="str">
         <f>IF('Filter Log'!A101="","",'Filter Log'!A101)</f>
         <v/>
       </c>
-      <c r="B101" s="21">
+      <c r="B101" s="21" t="str">
         <f>IF('Filter Log'!B101="","",'Filter Log'!B101)</f>
         <v/>
       </c>
-      <c r="C101" s="20">
+      <c r="C101" s="20" t="str">
         <f>IF('Filter Log'!C101="","",'Filter Log'!C101)</f>
         <v/>
       </c>
-      <c r="D101" s="20">
+      <c r="D101" s="20" t="str">
         <f>IF('Filter Log'!D101="","",'Filter Log'!D101)</f>
         <v/>
       </c>
-      <c r="E101" s="20">
+      <c r="E101" s="20" t="str">
         <f>IF('Filter Log'!E101="","",'Filter Log'!E101)</f>
         <v/>
       </c>
@@ -4796,23 +4796,23 @@
       <c r="G101" s="22" t="n"/>
     </row>
     <row r="102" ht="26" customHeight="1">
-      <c r="A102" s="20">
+      <c r="A102" s="20" t="str">
         <f>IF('Filter Log'!A102="","",'Filter Log'!A102)</f>
         <v/>
       </c>
-      <c r="B102" s="21">
+      <c r="B102" s="21" t="str">
         <f>IF('Filter Log'!B102="","",'Filter Log'!B102)</f>
         <v/>
       </c>
-      <c r="C102" s="20">
+      <c r="C102" s="20" t="str">
         <f>IF('Filter Log'!C102="","",'Filter Log'!C102)</f>
         <v/>
       </c>
-      <c r="D102" s="20">
+      <c r="D102" s="20" t="str">
         <f>IF('Filter Log'!D102="","",'Filter Log'!D102)</f>
         <v/>
       </c>
-      <c r="E102" s="20">
+      <c r="E102" s="20" t="str">
         <f>IF('Filter Log'!E102="","",'Filter Log'!E102)</f>
         <v/>
       </c>
@@ -4820,23 +4820,23 @@
       <c r="G102" s="22" t="n"/>
     </row>
     <row r="103" ht="26" customHeight="1">
-      <c r="A103" s="20">
+      <c r="A103" s="20" t="str">
         <f>IF('Filter Log'!A103="","",'Filter Log'!A103)</f>
         <v/>
       </c>
-      <c r="B103" s="21">
+      <c r="B103" s="21" t="str">
         <f>IF('Filter Log'!B103="","",'Filter Log'!B103)</f>
         <v/>
       </c>
-      <c r="C103" s="20">
+      <c r="C103" s="20" t="str">
         <f>IF('Filter Log'!C103="","",'Filter Log'!C103)</f>
         <v/>
       </c>
-      <c r="D103" s="20">
+      <c r="D103" s="20" t="str">
         <f>IF('Filter Log'!D103="","",'Filter Log'!D103)</f>
         <v/>
       </c>
-      <c r="E103" s="20">
+      <c r="E103" s="20" t="str">
         <f>IF('Filter Log'!E103="","",'Filter Log'!E103)</f>
         <v/>
       </c>
@@ -4844,23 +4844,23 @@
       <c r="G103" s="22" t="n"/>
     </row>
     <row r="104" ht="26" customHeight="1">
-      <c r="A104" s="20">
+      <c r="A104" s="20" t="str">
         <f>IF('Filter Log'!A104="","",'Filter Log'!A104)</f>
         <v/>
       </c>
-      <c r="B104" s="21">
+      <c r="B104" s="21" t="str">
         <f>IF('Filter Log'!B104="","",'Filter Log'!B104)</f>
         <v/>
       </c>
-      <c r="C104" s="20">
+      <c r="C104" s="20" t="str">
         <f>IF('Filter Log'!C104="","",'Filter Log'!C104)</f>
         <v/>
       </c>
-      <c r="D104" s="20">
+      <c r="D104" s="20" t="str">
         <f>IF('Filter Log'!D104="","",'Filter Log'!D104)</f>
         <v/>
       </c>
-      <c r="E104" s="20">
+      <c r="E104" s="20" t="str">
         <f>IF('Filter Log'!E104="","",'Filter Log'!E104)</f>
         <v/>
       </c>
@@ -4868,23 +4868,23 @@
       <c r="G104" s="22" t="n"/>
     </row>
     <row r="105" ht="26" customHeight="1">
-      <c r="A105" s="20">
+      <c r="A105" s="20" t="str">
         <f>IF('Filter Log'!A105="","",'Filter Log'!A105)</f>
         <v/>
       </c>
-      <c r="B105" s="21">
+      <c r="B105" s="21" t="str">
         <f>IF('Filter Log'!B105="","",'Filter Log'!B105)</f>
         <v/>
       </c>
-      <c r="C105" s="20">
+      <c r="C105" s="20" t="str">
         <f>IF('Filter Log'!C105="","",'Filter Log'!C105)</f>
         <v/>
       </c>
-      <c r="D105" s="20">
+      <c r="D105" s="20" t="str">
         <f>IF('Filter Log'!D105="","",'Filter Log'!D105)</f>
         <v/>
       </c>
-      <c r="E105" s="20">
+      <c r="E105" s="20" t="str">
         <f>IF('Filter Log'!E105="","",'Filter Log'!E105)</f>
         <v/>
       </c>
@@ -4892,23 +4892,23 @@
       <c r="G105" s="22" t="n"/>
     </row>
     <row r="106" ht="26" customHeight="1">
-      <c r="A106" s="20">
+      <c r="A106" s="20" t="str">
         <f>IF('Filter Log'!A106="","",'Filter Log'!A106)</f>
         <v/>
       </c>
-      <c r="B106" s="21">
+      <c r="B106" s="21" t="str">
         <f>IF('Filter Log'!B106="","",'Filter Log'!B106)</f>
         <v/>
       </c>
-      <c r="C106" s="20">
+      <c r="C106" s="20" t="str">
         <f>IF('Filter Log'!C106="","",'Filter Log'!C106)</f>
         <v/>
       </c>
-      <c r="D106" s="20">
+      <c r="D106" s="20" t="str">
         <f>IF('Filter Log'!D106="","",'Filter Log'!D106)</f>
         <v/>
       </c>
-      <c r="E106" s="20">
+      <c r="E106" s="20" t="str">
         <f>IF('Filter Log'!E106="","",'Filter Log'!E106)</f>
         <v/>
       </c>
@@ -4916,23 +4916,23 @@
       <c r="G106" s="22" t="n"/>
     </row>
     <row r="107" ht="26" customHeight="1">
-      <c r="A107" s="20">
+      <c r="A107" s="20" t="str">
         <f>IF('Filter Log'!A107="","",'Filter Log'!A107)</f>
         <v/>
       </c>
-      <c r="B107" s="21">
+      <c r="B107" s="21" t="str">
         <f>IF('Filter Log'!B107="","",'Filter Log'!B107)</f>
         <v/>
       </c>
-      <c r="C107" s="20">
+      <c r="C107" s="20" t="str">
         <f>IF('Filter Log'!C107="","",'Filter Log'!C107)</f>
         <v/>
       </c>
-      <c r="D107" s="20">
+      <c r="D107" s="20" t="str">
         <f>IF('Filter Log'!D107="","",'Filter Log'!D107)</f>
         <v/>
       </c>
-      <c r="E107" s="20">
+      <c r="E107" s="20" t="str">
         <f>IF('Filter Log'!E107="","",'Filter Log'!E107)</f>
         <v/>
       </c>
@@ -4940,23 +4940,23 @@
       <c r="G107" s="22" t="n"/>
     </row>
     <row r="108" ht="26" customHeight="1">
-      <c r="A108" s="20">
+      <c r="A108" s="20" t="str">
         <f>IF('Filter Log'!A108="","",'Filter Log'!A108)</f>
         <v/>
       </c>
-      <c r="B108" s="21">
+      <c r="B108" s="21" t="str">
         <f>IF('Filter Log'!B108="","",'Filter Log'!B108)</f>
         <v/>
       </c>
-      <c r="C108" s="20">
+      <c r="C108" s="20" t="str">
         <f>IF('Filter Log'!C108="","",'Filter Log'!C108)</f>
         <v/>
       </c>
-      <c r="D108" s="20">
+      <c r="D108" s="20" t="str">
         <f>IF('Filter Log'!D108="","",'Filter Log'!D108)</f>
         <v/>
       </c>
-      <c r="E108" s="20">
+      <c r="E108" s="20" t="str">
         <f>IF('Filter Log'!E108="","",'Filter Log'!E108)</f>
         <v/>
       </c>
@@ -4964,23 +4964,23 @@
       <c r="G108" s="22" t="n"/>
     </row>
     <row r="109" ht="26" customHeight="1">
-      <c r="A109" s="20">
+      <c r="A109" s="20" t="str">
         <f>IF('Filter Log'!A109="","",'Filter Log'!A109)</f>
         <v/>
       </c>
-      <c r="B109" s="21">
+      <c r="B109" s="21" t="str">
         <f>IF('Filter Log'!B109="","",'Filter Log'!B109)</f>
         <v/>
       </c>
-      <c r="C109" s="20">
+      <c r="C109" s="20" t="str">
         <f>IF('Filter Log'!C109="","",'Filter Log'!C109)</f>
         <v/>
       </c>
-      <c r="D109" s="20">
+      <c r="D109" s="20" t="str">
         <f>IF('Filter Log'!D109="","",'Filter Log'!D109)</f>
         <v/>
       </c>
-      <c r="E109" s="20">
+      <c r="E109" s="20" t="str">
         <f>IF('Filter Log'!E109="","",'Filter Log'!E109)</f>
         <v/>
       </c>
@@ -4988,23 +4988,23 @@
       <c r="G109" s="22" t="n"/>
     </row>
     <row r="110" ht="26" customHeight="1">
-      <c r="A110" s="20">
+      <c r="A110" s="20" t="str">
         <f>IF('Filter Log'!A110="","",'Filter Log'!A110)</f>
         <v/>
       </c>
-      <c r="B110" s="21">
+      <c r="B110" s="21" t="str">
         <f>IF('Filter Log'!B110="","",'Filter Log'!B110)</f>
         <v/>
       </c>
-      <c r="C110" s="20">
+      <c r="C110" s="20" t="str">
         <f>IF('Filter Log'!C110="","",'Filter Log'!C110)</f>
         <v/>
       </c>
-      <c r="D110" s="20">
+      <c r="D110" s="20" t="str">
         <f>IF('Filter Log'!D110="","",'Filter Log'!D110)</f>
         <v/>
       </c>
-      <c r="E110" s="20">
+      <c r="E110" s="20" t="str">
         <f>IF('Filter Log'!E110="","",'Filter Log'!E110)</f>
         <v/>
       </c>
@@ -5012,23 +5012,23 @@
       <c r="G110" s="22" t="n"/>
     </row>
     <row r="111" ht="26" customHeight="1">
-      <c r="A111" s="20">
+      <c r="A111" s="20" t="str">
         <f>IF('Filter Log'!A111="","",'Filter Log'!A111)</f>
         <v/>
       </c>
-      <c r="B111" s="21">
+      <c r="B111" s="21" t="str">
         <f>IF('Filter Log'!B111="","",'Filter Log'!B111)</f>
         <v/>
       </c>
-      <c r="C111" s="20">
+      <c r="C111" s="20" t="str">
         <f>IF('Filter Log'!C111="","",'Filter Log'!C111)</f>
         <v/>
       </c>
-      <c r="D111" s="20">
+      <c r="D111" s="20" t="str">
         <f>IF('Filter Log'!D111="","",'Filter Log'!D111)</f>
         <v/>
       </c>
-      <c r="E111" s="20">
+      <c r="E111" s="20" t="str">
         <f>IF('Filter Log'!E111="","",'Filter Log'!E111)</f>
         <v/>
       </c>
@@ -5036,23 +5036,23 @@
       <c r="G111" s="22" t="n"/>
     </row>
     <row r="112" ht="26" customHeight="1">
-      <c r="A112" s="20">
+      <c r="A112" s="20" t="str">
         <f>IF('Filter Log'!A112="","",'Filter Log'!A112)</f>
         <v/>
       </c>
-      <c r="B112" s="21">
+      <c r="B112" s="21" t="str">
         <f>IF('Filter Log'!B112="","",'Filter Log'!B112)</f>
         <v/>
       </c>
-      <c r="C112" s="20">
+      <c r="C112" s="20" t="str">
         <f>IF('Filter Log'!C112="","",'Filter Log'!C112)</f>
         <v/>
       </c>
-      <c r="D112" s="20">
+      <c r="D112" s="20" t="str">
         <f>IF('Filter Log'!D112="","",'Filter Log'!D112)</f>
         <v/>
       </c>
-      <c r="E112" s="20">
+      <c r="E112" s="20" t="str">
         <f>IF('Filter Log'!E112="","",'Filter Log'!E112)</f>
         <v/>
       </c>
@@ -5060,23 +5060,23 @@
       <c r="G112" s="22" t="n"/>
     </row>
     <row r="113" ht="26" customHeight="1">
-      <c r="A113" s="20">
+      <c r="A113" s="20" t="str">
         <f>IF('Filter Log'!A113="","",'Filter Log'!A113)</f>
         <v/>
       </c>
-      <c r="B113" s="21">
+      <c r="B113" s="21" t="str">
         <f>IF('Filter Log'!B113="","",'Filter Log'!B113)</f>
         <v/>
       </c>
-      <c r="C113" s="20">
+      <c r="C113" s="20" t="str">
         <f>IF('Filter Log'!C113="","",'Filter Log'!C113)</f>
         <v/>
       </c>
-      <c r="D113" s="20">
+      <c r="D113" s="20" t="str">
         <f>IF('Filter Log'!D113="","",'Filter Log'!D113)</f>
         <v/>
       </c>
-      <c r="E113" s="20">
+      <c r="E113" s="20" t="str">
         <f>IF('Filter Log'!E113="","",'Filter Log'!E113)</f>
         <v/>
       </c>
@@ -5084,23 +5084,23 @@
       <c r="G113" s="22" t="n"/>
     </row>
     <row r="114" ht="26" customHeight="1">
-      <c r="A114" s="20">
+      <c r="A114" s="20" t="str">
         <f>IF('Filter Log'!A114="","",'Filter Log'!A114)</f>
         <v/>
       </c>
-      <c r="B114" s="21">
+      <c r="B114" s="21" t="str">
         <f>IF('Filter Log'!B114="","",'Filter Log'!B114)</f>
         <v/>
       </c>
-      <c r="C114" s="20">
+      <c r="C114" s="20" t="str">
         <f>IF('Filter Log'!C114="","",'Filter Log'!C114)</f>
         <v/>
       </c>
-      <c r="D114" s="20">
+      <c r="D114" s="20" t="str">
         <f>IF('Filter Log'!D114="","",'Filter Log'!D114)</f>
         <v/>
       </c>
-      <c r="E114" s="20">
+      <c r="E114" s="20" t="str">
         <f>IF('Filter Log'!E114="","",'Filter Log'!E114)</f>
         <v/>
       </c>
@@ -5108,23 +5108,23 @@
       <c r="G114" s="22" t="n"/>
     </row>
     <row r="115" ht="26" customHeight="1">
-      <c r="A115" s="20">
+      <c r="A115" s="20" t="str">
         <f>IF('Filter Log'!A115="","",'Filter Log'!A115)</f>
         <v/>
       </c>
-      <c r="B115" s="21">
+      <c r="B115" s="21" t="str">
         <f>IF('Filter Log'!B115="","",'Filter Log'!B115)</f>
         <v/>
       </c>
-      <c r="C115" s="20">
+      <c r="C115" s="20" t="str">
         <f>IF('Filter Log'!C115="","",'Filter Log'!C115)</f>
         <v/>
       </c>
-      <c r="D115" s="20">
+      <c r="D115" s="20" t="str">
         <f>IF('Filter Log'!D115="","",'Filter Log'!D115)</f>
         <v/>
       </c>
-      <c r="E115" s="20">
+      <c r="E115" s="20" t="str">
         <f>IF('Filter Log'!E115="","",'Filter Log'!E115)</f>
         <v/>
       </c>
@@ -5132,23 +5132,23 @@
       <c r="G115" s="22" t="n"/>
     </row>
     <row r="116" ht="26" customHeight="1">
-      <c r="A116" s="20">
+      <c r="A116" s="20" t="str">
         <f>IF('Filter Log'!A116="","",'Filter Log'!A116)</f>
         <v/>
       </c>
-      <c r="B116" s="21">
+      <c r="B116" s="21" t="str">
         <f>IF('Filter Log'!B116="","",'Filter Log'!B116)</f>
         <v/>
       </c>
-      <c r="C116" s="20">
+      <c r="C116" s="20" t="str">
         <f>IF('Filter Log'!C116="","",'Filter Log'!C116)</f>
         <v/>
       </c>
-      <c r="D116" s="20">
+      <c r="D116" s="20" t="str">
         <f>IF('Filter Log'!D116="","",'Filter Log'!D116)</f>
         <v/>
       </c>
-      <c r="E116" s="20">
+      <c r="E116" s="20" t="str">
         <f>IF('Filter Log'!E116="","",'Filter Log'!E116)</f>
         <v/>
       </c>
@@ -5156,23 +5156,23 @@
       <c r="G116" s="22" t="n"/>
     </row>
     <row r="117" ht="26" customHeight="1">
-      <c r="A117" s="20">
+      <c r="A117" s="20" t="str">
         <f>IF('Filter Log'!A117="","",'Filter Log'!A117)</f>
         <v/>
       </c>
-      <c r="B117" s="21">
+      <c r="B117" s="21" t="str">
         <f>IF('Filter Log'!B117="","",'Filter Log'!B117)</f>
         <v/>
       </c>
-      <c r="C117" s="20">
+      <c r="C117" s="20" t="str">
         <f>IF('Filter Log'!C117="","",'Filter Log'!C117)</f>
         <v/>
       </c>
-      <c r="D117" s="20">
+      <c r="D117" s="20" t="str">
         <f>IF('Filter Log'!D117="","",'Filter Log'!D117)</f>
         <v/>
       </c>
-      <c r="E117" s="20">
+      <c r="E117" s="20" t="str">
         <f>IF('Filter Log'!E117="","",'Filter Log'!E117)</f>
         <v/>
       </c>
@@ -5180,23 +5180,23 @@
       <c r="G117" s="22" t="n"/>
     </row>
     <row r="118" ht="26" customHeight="1">
-      <c r="A118" s="20">
+      <c r="A118" s="20" t="str">
         <f>IF('Filter Log'!A118="","",'Filter Log'!A118)</f>
         <v/>
       </c>
-      <c r="B118" s="21">
+      <c r="B118" s="21" t="str">
         <f>IF('Filter Log'!B118="","",'Filter Log'!B118)</f>
         <v/>
       </c>
-      <c r="C118" s="20">
+      <c r="C118" s="20" t="str">
         <f>IF('Filter Log'!C118="","",'Filter Log'!C118)</f>
         <v/>
       </c>
-      <c r="D118" s="20">
+      <c r="D118" s="20" t="str">
         <f>IF('Filter Log'!D118="","",'Filter Log'!D118)</f>
         <v/>
       </c>
-      <c r="E118" s="20">
+      <c r="E118" s="20" t="str">
         <f>IF('Filter Log'!E118="","",'Filter Log'!E118)</f>
         <v/>
       </c>
@@ -5204,23 +5204,23 @@
       <c r="G118" s="22" t="n"/>
     </row>
     <row r="119" ht="26" customHeight="1">
-      <c r="A119" s="20">
+      <c r="A119" s="20" t="str">
         <f>IF('Filter Log'!A119="","",'Filter Log'!A119)</f>
         <v/>
       </c>
-      <c r="B119" s="21">
+      <c r="B119" s="21" t="str">
         <f>IF('Filter Log'!B119="","",'Filter Log'!B119)</f>
         <v/>
       </c>
-      <c r="C119" s="20">
+      <c r="C119" s="20" t="str">
         <f>IF('Filter Log'!C119="","",'Filter Log'!C119)</f>
         <v/>
       </c>
-      <c r="D119" s="20">
+      <c r="D119" s="20" t="str">
         <f>IF('Filter Log'!D119="","",'Filter Log'!D119)</f>
         <v/>
       </c>
-      <c r="E119" s="20">
+      <c r="E119" s="20" t="str">
         <f>IF('Filter Log'!E119="","",'Filter Log'!E119)</f>
         <v/>
       </c>
@@ -5228,23 +5228,23 @@
       <c r="G119" s="22" t="n"/>
     </row>
     <row r="120" ht="26" customHeight="1">
-      <c r="A120" s="20">
+      <c r="A120" s="20" t="str">
         <f>IF('Filter Log'!A120="","",'Filter Log'!A120)</f>
         <v/>
       </c>
-      <c r="B120" s="21">
+      <c r="B120" s="21" t="str">
         <f>IF('Filter Log'!B120="","",'Filter Log'!B120)</f>
         <v/>
       </c>
-      <c r="C120" s="20">
+      <c r="C120" s="20" t="str">
         <f>IF('Filter Log'!C120="","",'Filter Log'!C120)</f>
         <v/>
       </c>
-      <c r="D120" s="20">
+      <c r="D120" s="20" t="str">
         <f>IF('Filter Log'!D120="","",'Filter Log'!D120)</f>
         <v/>
       </c>
-      <c r="E120" s="20">
+      <c r="E120" s="20" t="str">
         <f>IF('Filter Log'!E120="","",'Filter Log'!E120)</f>
         <v/>
       </c>
@@ -5252,23 +5252,23 @@
       <c r="G120" s="22" t="n"/>
     </row>
     <row r="121" ht="26" customHeight="1">
-      <c r="A121" s="20">
+      <c r="A121" s="20" t="str">
         <f>IF('Filter Log'!A121="","",'Filter Log'!A121)</f>
         <v/>
       </c>
-      <c r="B121" s="21">
+      <c r="B121" s="21" t="str">
         <f>IF('Filter Log'!B121="","",'Filter Log'!B121)</f>
         <v/>
       </c>
-      <c r="C121" s="20">
+      <c r="C121" s="20" t="str">
         <f>IF('Filter Log'!C121="","",'Filter Log'!C121)</f>
         <v/>
       </c>
-      <c r="D121" s="20">
+      <c r="D121" s="20" t="str">
         <f>IF('Filter Log'!D121="","",'Filter Log'!D121)</f>
         <v/>
       </c>
-      <c r="E121" s="20">
+      <c r="E121" s="20" t="str">
         <f>IF('Filter Log'!E121="","",'Filter Log'!E121)</f>
         <v/>
       </c>
@@ -5276,23 +5276,23 @@
       <c r="G121" s="22" t="n"/>
     </row>
     <row r="122" ht="26" customHeight="1">
-      <c r="A122" s="20">
+      <c r="A122" s="20" t="str">
         <f>IF('Filter Log'!A122="","",'Filter Log'!A122)</f>
         <v/>
       </c>
-      <c r="B122" s="21">
+      <c r="B122" s="21" t="str">
         <f>IF('Filter Log'!B122="","",'Filter Log'!B122)</f>
         <v/>
       </c>
-      <c r="C122" s="20">
+      <c r="C122" s="20" t="str">
         <f>IF('Filter Log'!C122="","",'Filter Log'!C122)</f>
         <v/>
       </c>
-      <c r="D122" s="20">
+      <c r="D122" s="20" t="str">
         <f>IF('Filter Log'!D122="","",'Filter Log'!D122)</f>
         <v/>
       </c>
-      <c r="E122" s="20">
+      <c r="E122" s="20" t="str">
         <f>IF('Filter Log'!E122="","",'Filter Log'!E122)</f>
         <v/>
       </c>
@@ -5300,23 +5300,23 @@
       <c r="G122" s="22" t="n"/>
     </row>
     <row r="123" ht="26" customHeight="1">
-      <c r="A123" s="20">
+      <c r="A123" s="20" t="str">
         <f>IF('Filter Log'!A123="","",'Filter Log'!A123)</f>
         <v/>
       </c>
-      <c r="B123" s="21">
+      <c r="B123" s="21" t="str">
         <f>IF('Filter Log'!B123="","",'Filter Log'!B123)</f>
         <v/>
       </c>
-      <c r="C123" s="20">
+      <c r="C123" s="20" t="str">
         <f>IF('Filter Log'!C123="","",'Filter Log'!C123)</f>
         <v/>
       </c>
-      <c r="D123" s="20">
+      <c r="D123" s="20" t="str">
         <f>IF('Filter Log'!D123="","",'Filter Log'!D123)</f>
         <v/>
       </c>
-      <c r="E123" s="20">
+      <c r="E123" s="20" t="str">
         <f>IF('Filter Log'!E123="","",'Filter Log'!E123)</f>
         <v/>
       </c>
@@ -5324,23 +5324,23 @@
       <c r="G123" s="22" t="n"/>
     </row>
     <row r="124" ht="26" customHeight="1">
-      <c r="A124" s="20">
+      <c r="A124" s="20" t="str">
         <f>IF('Filter Log'!A124="","",'Filter Log'!A124)</f>
         <v/>
       </c>
-      <c r="B124" s="21">
+      <c r="B124" s="21" t="str">
         <f>IF('Filter Log'!B124="","",'Filter Log'!B124)</f>
         <v/>
       </c>
-      <c r="C124" s="20">
+      <c r="C124" s="20" t="str">
         <f>IF('Filter Log'!C124="","",'Filter Log'!C124)</f>
         <v/>
       </c>
-      <c r="D124" s="20">
+      <c r="D124" s="20" t="str">
         <f>IF('Filter Log'!D124="","",'Filter Log'!D124)</f>
         <v/>
       </c>
-      <c r="E124" s="20">
+      <c r="E124" s="20" t="str">
         <f>IF('Filter Log'!E124="","",'Filter Log'!E124)</f>
         <v/>
       </c>
@@ -5426,7 +5426,7 @@
           <t>Job number</t>
         </is>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="4" t="str">
         <f>IF('Filter Log'!B2="","",'Filter Log'!B2)</f>
         <v/>
       </c>
@@ -5440,7 +5440,7 @@
           <t>Airco PM</t>
         </is>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="4" t="str">
         <f>IF('Filter Log'!I2="","",'Filter Log'!I2)</f>
         <v/>
       </c>
@@ -5456,7 +5456,7 @@
           <t>Project name</t>
         </is>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="9" t="str">
         <f>IF('Filter Log'!B3="","",'Filter Log'!B3)</f>
         <v/>
       </c>
@@ -5470,7 +5470,7 @@
           <t>Airco APM</t>
         </is>
       </c>
-      <c r="I3" s="9">
+      <c r="I3" s="9" t="str">
         <f>IF('Filter Log'!I3="","",'Filter Log'!I3)</f>
         <v/>
       </c>
@@ -5486,7 +5486,7 @@
           <t>Phase</t>
         </is>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="9" t="str">
         <f>IF('Filter Log'!B4="","",'Filter Log'!B4)</f>
         <v/>
       </c>
@@ -5500,7 +5500,7 @@
           <t>GC</t>
         </is>
       </c>
-      <c r="I4" s="9">
+      <c r="I4" s="9" t="str">
         <f>IF('Filter Log'!I4="","",'Filter Log'!I4)</f>
         <v/>
       </c>
@@ -5516,7 +5516,7 @@
           <t>Job type</t>
         </is>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="9" t="str">
         <f>IF('Filter Log'!B5="","",'Filter Log'!B5)</f>
         <v/>
       </c>
@@ -5611,7 +5611,7 @@
       <c r="I8" s="14" t="n"/>
       <c r="J8" s="14" t="n"/>
       <c r="K8" s="23" t="n"/>
-      <c r="L8" s="23">
+      <c r="L8" s="23" t="str">
         <f>IF(OR(J8="",K8=""),"",J8*K8)</f>
         <v/>
       </c>
@@ -5630,7 +5630,7 @@
       <c r="I9" s="14" t="n"/>
       <c r="J9" s="14" t="n"/>
       <c r="K9" s="23" t="n"/>
-      <c r="L9" s="23">
+      <c r="L9" s="23" t="str">
         <f>IF(OR(J9="",K9=""),"",J9*K9)</f>
         <v/>
       </c>
@@ -5649,7 +5649,7 @@
       <c r="I10" s="14" t="n"/>
       <c r="J10" s="14" t="n"/>
       <c r="K10" s="23" t="n"/>
-      <c r="L10" s="23">
+      <c r="L10" s="23" t="str">
         <f>IF(OR(J10="",K10=""),"",J10*K10)</f>
         <v/>
       </c>
@@ -5668,7 +5668,7 @@
       <c r="I11" s="14" t="n"/>
       <c r="J11" s="14" t="n"/>
       <c r="K11" s="23" t="n"/>
-      <c r="L11" s="23">
+      <c r="L11" s="23" t="str">
         <f>IF(OR(J11="",K11=""),"",J11*K11)</f>
         <v/>
       </c>
@@ -5687,7 +5687,7 @@
       <c r="I12" s="14" t="n"/>
       <c r="J12" s="14" t="n"/>
       <c r="K12" s="23" t="n"/>
-      <c r="L12" s="23">
+      <c r="L12" s="23" t="str">
         <f>IF(OR(J12="",K12=""),"",J12*K12)</f>
         <v/>
       </c>
@@ -5706,7 +5706,7 @@
       <c r="I13" s="14" t="n"/>
       <c r="J13" s="14" t="n"/>
       <c r="K13" s="23" t="n"/>
-      <c r="L13" s="23">
+      <c r="L13" s="23" t="str">
         <f>IF(OR(J13="",K13=""),"",J13*K13)</f>
         <v/>
       </c>
@@ -5725,7 +5725,7 @@
       <c r="I14" s="14" t="n"/>
       <c r="J14" s="14" t="n"/>
       <c r="K14" s="23" t="n"/>
-      <c r="L14" s="23">
+      <c r="L14" s="23" t="str">
         <f>IF(OR(J14="",K14=""),"",J14*K14)</f>
         <v/>
       </c>
@@ -5744,7 +5744,7 @@
       <c r="I15" s="14" t="n"/>
       <c r="J15" s="14" t="n"/>
       <c r="K15" s="23" t="n"/>
-      <c r="L15" s="23">
+      <c r="L15" s="23" t="str">
         <f>IF(OR(J15="",K15=""),"",J15*K15)</f>
         <v/>
       </c>
@@ -5763,7 +5763,7 @@
       <c r="I16" s="14" t="n"/>
       <c r="J16" s="14" t="n"/>
       <c r="K16" s="23" t="n"/>
-      <c r="L16" s="23">
+      <c r="L16" s="23" t="str">
         <f>IF(OR(J16="",K16=""),"",J16*K16)</f>
         <v/>
       </c>
@@ -5782,7 +5782,7 @@
       <c r="I17" s="14" t="n"/>
       <c r="J17" s="14" t="n"/>
       <c r="K17" s="23" t="n"/>
-      <c r="L17" s="23">
+      <c r="L17" s="23" t="str">
         <f>IF(OR(J17="",K17=""),"",J17*K17)</f>
         <v/>
       </c>
@@ -5801,7 +5801,7 @@
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="14" t="n"/>
       <c r="K18" s="23" t="n"/>
-      <c r="L18" s="23">
+      <c r="L18" s="23" t="str">
         <f>IF(OR(J18="",K18=""),"",J18*K18)</f>
         <v/>
       </c>
@@ -5820,7 +5820,7 @@
       <c r="I19" s="14" t="n"/>
       <c r="J19" s="14" t="n"/>
       <c r="K19" s="23" t="n"/>
-      <c r="L19" s="23">
+      <c r="L19" s="23" t="str">
         <f>IF(OR(J19="",K19=""),"",J19*K19)</f>
         <v/>
       </c>
@@ -5839,7 +5839,7 @@
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="14" t="n"/>
       <c r="K20" s="23" t="n"/>
-      <c r="L20" s="23">
+      <c r="L20" s="23" t="str">
         <f>IF(OR(J20="",K20=""),"",J20*K20)</f>
         <v/>
       </c>
@@ -5858,7 +5858,7 @@
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="14" t="n"/>
       <c r="K21" s="23" t="n"/>
-      <c r="L21" s="23">
+      <c r="L21" s="23" t="str">
         <f>IF(OR(J21="",K21=""),"",J21*K21)</f>
         <v/>
       </c>
@@ -5877,7 +5877,7 @@
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="14" t="n"/>
       <c r="K22" s="23" t="n"/>
-      <c r="L22" s="23">
+      <c r="L22" s="23" t="str">
         <f>IF(OR(J22="",K22=""),"",J22*K22)</f>
         <v/>
       </c>
@@ -5896,7 +5896,7 @@
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="14" t="n"/>
       <c r="K23" s="23" t="n"/>
-      <c r="L23" s="23">
+      <c r="L23" s="23" t="str">
         <f>IF(OR(J23="",K23=""),"",J23*K23)</f>
         <v/>
       </c>
@@ -5915,7 +5915,7 @@
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="14" t="n"/>
       <c r="K24" s="23" t="n"/>
-      <c r="L24" s="23">
+      <c r="L24" s="23" t="str">
         <f>IF(OR(J24="",K24=""),"",J24*K24)</f>
         <v/>
       </c>
@@ -5934,7 +5934,7 @@
       <c r="I25" s="14" t="n"/>
       <c r="J25" s="14" t="n"/>
       <c r="K25" s="23" t="n"/>
-      <c r="L25" s="23">
+      <c r="L25" s="23" t="str">
         <f>IF(OR(J25="",K25=""),"",J25*K25)</f>
         <v/>
       </c>
@@ -5953,7 +5953,7 @@
       <c r="I26" s="14" t="n"/>
       <c r="J26" s="14" t="n"/>
       <c r="K26" s="23" t="n"/>
-      <c r="L26" s="23">
+      <c r="L26" s="23" t="str">
         <f>IF(OR(J26="",K26=""),"",J26*K26)</f>
         <v/>
       </c>
@@ -5972,7 +5972,7 @@
       <c r="I27" s="14" t="n"/>
       <c r="J27" s="14" t="n"/>
       <c r="K27" s="23" t="n"/>
-      <c r="L27" s="23">
+      <c r="L27" s="23" t="str">
         <f>IF(OR(J27="",K27=""),"",J27*K27)</f>
         <v/>
       </c>
@@ -5991,7 +5991,7 @@
       <c r="I28" s="14" t="n"/>
       <c r="J28" s="14" t="n"/>
       <c r="K28" s="23" t="n"/>
-      <c r="L28" s="23">
+      <c r="L28" s="23" t="str">
         <f>IF(OR(J28="",K28=""),"",J28*K28)</f>
         <v/>
       </c>
@@ -6010,7 +6010,7 @@
       <c r="I29" s="14" t="n"/>
       <c r="J29" s="14" t="n"/>
       <c r="K29" s="23" t="n"/>
-      <c r="L29" s="23">
+      <c r="L29" s="23" t="str">
         <f>IF(OR(J29="",K29=""),"",J29*K29)</f>
         <v/>
       </c>
@@ -6029,7 +6029,7 @@
       <c r="I30" s="14" t="n"/>
       <c r="J30" s="14" t="n"/>
       <c r="K30" s="23" t="n"/>
-      <c r="L30" s="23">
+      <c r="L30" s="23" t="str">
         <f>IF(OR(J30="",K30=""),"",J30*K30)</f>
         <v/>
       </c>
@@ -6048,7 +6048,7 @@
       <c r="I31" s="14" t="n"/>
       <c r="J31" s="14" t="n"/>
       <c r="K31" s="23" t="n"/>
-      <c r="L31" s="23">
+      <c r="L31" s="23" t="str">
         <f>IF(OR(J31="",K31=""),"",J31*K31)</f>
         <v/>
       </c>
@@ -6067,7 +6067,7 @@
       <c r="I32" s="14" t="n"/>
       <c r="J32" s="14" t="n"/>
       <c r="K32" s="23" t="n"/>
-      <c r="L32" s="23">
+      <c r="L32" s="23" t="str">
         <f>IF(OR(J32="",K32=""),"",J32*K32)</f>
         <v/>
       </c>
@@ -6086,7 +6086,7 @@
       <c r="I33" s="14" t="n"/>
       <c r="J33" s="14" t="n"/>
       <c r="K33" s="23" t="n"/>
-      <c r="L33" s="23">
+      <c r="L33" s="23" t="str">
         <f>IF(OR(J33="",K33=""),"",J33*K33)</f>
         <v/>
       </c>
@@ -6105,7 +6105,7 @@
       <c r="I34" s="14" t="n"/>
       <c r="J34" s="14" t="n"/>
       <c r="K34" s="23" t="n"/>
-      <c r="L34" s="23">
+      <c r="L34" s="23" t="str">
         <f>IF(OR(J34="",K34=""),"",J34*K34)</f>
         <v/>
       </c>
@@ -6124,7 +6124,7 @@
       <c r="I35" s="14" t="n"/>
       <c r="J35" s="14" t="n"/>
       <c r="K35" s="23" t="n"/>
-      <c r="L35" s="23">
+      <c r="L35" s="23" t="str">
         <f>IF(OR(J35="",K35=""),"",J35*K35)</f>
         <v/>
       </c>
@@ -6143,7 +6143,7 @@
       <c r="I36" s="14" t="n"/>
       <c r="J36" s="14" t="n"/>
       <c r="K36" s="23" t="n"/>
-      <c r="L36" s="23">
+      <c r="L36" s="23" t="str">
         <f>IF(OR(J36="",K36=""),"",J36*K36)</f>
         <v/>
       </c>
@@ -6162,7 +6162,7 @@
       <c r="I37" s="14" t="n"/>
       <c r="J37" s="14" t="n"/>
       <c r="K37" s="23" t="n"/>
-      <c r="L37" s="23">
+      <c r="L37" s="23" t="str">
         <f>IF(OR(J37="",K37=""),"",J37*K37)</f>
         <v/>
       </c>
@@ -6181,7 +6181,7 @@
       <c r="I38" s="14" t="n"/>
       <c r="J38" s="14" t="n"/>
       <c r="K38" s="23" t="n"/>
-      <c r="L38" s="23">
+      <c r="L38" s="23" t="str">
         <f>IF(OR(J38="",K38=""),"",J38*K38)</f>
         <v/>
       </c>
@@ -6200,7 +6200,7 @@
       <c r="I39" s="14" t="n"/>
       <c r="J39" s="14" t="n"/>
       <c r="K39" s="23" t="n"/>
-      <c r="L39" s="23">
+      <c r="L39" s="23" t="str">
         <f>IF(OR(J39="",K39=""),"",J39*K39)</f>
         <v/>
       </c>
@@ -6219,7 +6219,7 @@
       <c r="I40" s="14" t="n"/>
       <c r="J40" s="14" t="n"/>
       <c r="K40" s="23" t="n"/>
-      <c r="L40" s="23">
+      <c r="L40" s="23" t="str">
         <f>IF(OR(J40="",K40=""),"",J40*K40)</f>
         <v/>
       </c>
@@ -6238,7 +6238,7 @@
       <c r="I41" s="14" t="n"/>
       <c r="J41" s="14" t="n"/>
       <c r="K41" s="23" t="n"/>
-      <c r="L41" s="23">
+      <c r="L41" s="23" t="str">
         <f>IF(OR(J41="",K41=""),"",J41*K41)</f>
         <v/>
       </c>
@@ -6257,7 +6257,7 @@
       <c r="I42" s="14" t="n"/>
       <c r="J42" s="14" t="n"/>
       <c r="K42" s="23" t="n"/>
-      <c r="L42" s="23">
+      <c r="L42" s="23" t="str">
         <f>IF(OR(J42="",K42=""),"",J42*K42)</f>
         <v/>
       </c>
@@ -6276,7 +6276,7 @@
       <c r="I43" s="14" t="n"/>
       <c r="J43" s="14" t="n"/>
       <c r="K43" s="23" t="n"/>
-      <c r="L43" s="23">
+      <c r="L43" s="23" t="str">
         <f>IF(OR(J43="",K43=""),"",J43*K43)</f>
         <v/>
       </c>
@@ -6295,7 +6295,7 @@
       <c r="I44" s="14" t="n"/>
       <c r="J44" s="14" t="n"/>
       <c r="K44" s="23" t="n"/>
-      <c r="L44" s="23">
+      <c r="L44" s="23" t="str">
         <f>IF(OR(J44="",K44=""),"",J44*K44)</f>
         <v/>
       </c>
@@ -6314,7 +6314,7 @@
       <c r="I45" s="14" t="n"/>
       <c r="J45" s="14" t="n"/>
       <c r="K45" s="23" t="n"/>
-      <c r="L45" s="23">
+      <c r="L45" s="23" t="str">
         <f>IF(OR(J45="",K45=""),"",J45*K45)</f>
         <v/>
       </c>
@@ -6333,7 +6333,7 @@
       <c r="I46" s="14" t="n"/>
       <c r="J46" s="14" t="n"/>
       <c r="K46" s="23" t="n"/>
-      <c r="L46" s="23">
+      <c r="L46" s="23" t="str">
         <f>IF(OR(J46="",K46=""),"",J46*K46)</f>
         <v/>
       </c>
@@ -6352,7 +6352,7 @@
       <c r="I47" s="14" t="n"/>
       <c r="J47" s="14" t="n"/>
       <c r="K47" s="23" t="n"/>
-      <c r="L47" s="23">
+      <c r="L47" s="23" t="str">
         <f>IF(OR(J47="",K47=""),"",J47*K47)</f>
         <v/>
       </c>
@@ -6371,7 +6371,7 @@
       <c r="I48" s="14" t="n"/>
       <c r="J48" s="14" t="n"/>
       <c r="K48" s="23" t="n"/>
-      <c r="L48" s="23">
+      <c r="L48" s="23" t="str">
         <f>IF(OR(J48="",K48=""),"",J48*K48)</f>
         <v/>
       </c>
@@ -6390,7 +6390,7 @@
       <c r="I49" s="14" t="n"/>
       <c r="J49" s="14" t="n"/>
       <c r="K49" s="23" t="n"/>
-      <c r="L49" s="23">
+      <c r="L49" s="23" t="str">
         <f>IF(OR(J49="",K49=""),"",J49*K49)</f>
         <v/>
       </c>
@@ -6409,7 +6409,7 @@
       <c r="I50" s="14" t="n"/>
       <c r="J50" s="14" t="n"/>
       <c r="K50" s="23" t="n"/>
-      <c r="L50" s="23">
+      <c r="L50" s="23" t="str">
         <f>IF(OR(J50="",K50=""),"",J50*K50)</f>
         <v/>
       </c>
@@ -6428,7 +6428,7 @@
       <c r="I51" s="14" t="n"/>
       <c r="J51" s="14" t="n"/>
       <c r="K51" s="23" t="n"/>
-      <c r="L51" s="23">
+      <c r="L51" s="23" t="str">
         <f>IF(OR(J51="",K51=""),"",J51*K51)</f>
         <v/>
       </c>
@@ -6447,7 +6447,7 @@
       <c r="I52" s="14" t="n"/>
       <c r="J52" s="14" t="n"/>
       <c r="K52" s="23" t="n"/>
-      <c r="L52" s="23">
+      <c r="L52" s="23" t="str">
         <f>IF(OR(J52="",K52=""),"",J52*K52)</f>
         <v/>
       </c>
@@ -6466,7 +6466,7 @@
       <c r="I53" s="14" t="n"/>
       <c r="J53" s="14" t="n"/>
       <c r="K53" s="23" t="n"/>
-      <c r="L53" s="23">
+      <c r="L53" s="23" t="str">
         <f>IF(OR(J53="",K53=""),"",J53*K53)</f>
         <v/>
       </c>
@@ -6485,7 +6485,7 @@
       <c r="I54" s="14" t="n"/>
       <c r="J54" s="14" t="n"/>
       <c r="K54" s="23" t="n"/>
-      <c r="L54" s="23">
+      <c r="L54" s="23" t="str">
         <f>IF(OR(J54="",K54=""),"",J54*K54)</f>
         <v/>
       </c>
@@ -6504,7 +6504,7 @@
       <c r="I55" s="14" t="n"/>
       <c r="J55" s="14" t="n"/>
       <c r="K55" s="23" t="n"/>
-      <c r="L55" s="23">
+      <c r="L55" s="23" t="str">
         <f>IF(OR(J55="",K55=""),"",J55*K55)</f>
         <v/>
       </c>
@@ -6523,7 +6523,7 @@
       <c r="I56" s="14" t="n"/>
       <c r="J56" s="14" t="n"/>
       <c r="K56" s="23" t="n"/>
-      <c r="L56" s="23">
+      <c r="L56" s="23" t="str">
         <f>IF(OR(J56="",K56=""),"",J56*K56)</f>
         <v/>
       </c>
@@ -6542,7 +6542,7 @@
       <c r="I57" s="14" t="n"/>
       <c r="J57" s="14" t="n"/>
       <c r="K57" s="23" t="n"/>
-      <c r="L57" s="23">
+      <c r="L57" s="23" t="str">
         <f>IF(OR(J57="",K57=""),"",J57*K57)</f>
         <v/>
       </c>
@@ -6561,7 +6561,7 @@
       <c r="I58" s="14" t="n"/>
       <c r="J58" s="14" t="n"/>
       <c r="K58" s="23" t="n"/>
-      <c r="L58" s="23">
+      <c r="L58" s="23" t="str">
         <f>IF(OR(J58="",K58=""),"",J58*K58)</f>
         <v/>
       </c>
@@ -6580,7 +6580,7 @@
       <c r="I59" s="14" t="n"/>
       <c r="J59" s="14" t="n"/>
       <c r="K59" s="23" t="n"/>
-      <c r="L59" s="23">
+      <c r="L59" s="23" t="str">
         <f>IF(OR(J59="",K59=""),"",J59*K59)</f>
         <v/>
       </c>
@@ -6599,7 +6599,7 @@
       <c r="I60" s="14" t="n"/>
       <c r="J60" s="14" t="n"/>
       <c r="K60" s="23" t="n"/>
-      <c r="L60" s="23">
+      <c r="L60" s="23" t="str">
         <f>IF(OR(J60="",K60=""),"",J60*K60)</f>
         <v/>
       </c>
@@ -6618,7 +6618,7 @@
       <c r="I61" s="14" t="n"/>
       <c r="J61" s="14" t="n"/>
       <c r="K61" s="23" t="n"/>
-      <c r="L61" s="23">
+      <c r="L61" s="23" t="str">
         <f>IF(OR(J61="",K61=""),"",J61*K61)</f>
         <v/>
       </c>
@@ -6637,7 +6637,7 @@
       <c r="I62" s="14" t="n"/>
       <c r="J62" s="14" t="n"/>
       <c r="K62" s="23" t="n"/>
-      <c r="L62" s="23">
+      <c r="L62" s="23" t="str">
         <f>IF(OR(J62="",K62=""),"",J62*K62)</f>
         <v/>
       </c>
@@ -6656,7 +6656,7 @@
       <c r="I63" s="14" t="n"/>
       <c r="J63" s="14" t="n"/>
       <c r="K63" s="23" t="n"/>
-      <c r="L63" s="23">
+      <c r="L63" s="23" t="str">
         <f>IF(OR(J63="",K63=""),"",J63*K63)</f>
         <v/>
       </c>
@@ -6675,7 +6675,7 @@
       <c r="I64" s="14" t="n"/>
       <c r="J64" s="14" t="n"/>
       <c r="K64" s="23" t="n"/>
-      <c r="L64" s="23">
+      <c r="L64" s="23" t="str">
         <f>IF(OR(J64="",K64=""),"",J64*K64)</f>
         <v/>
       </c>
@@ -6694,7 +6694,7 @@
       <c r="I65" s="14" t="n"/>
       <c r="J65" s="14" t="n"/>
       <c r="K65" s="23" t="n"/>
-      <c r="L65" s="23">
+      <c r="L65" s="23" t="str">
         <f>IF(OR(J65="",K65=""),"",J65*K65)</f>
         <v/>
       </c>
@@ -6713,7 +6713,7 @@
       <c r="I66" s="14" t="n"/>
       <c r="J66" s="14" t="n"/>
       <c r="K66" s="23" t="n"/>
-      <c r="L66" s="23">
+      <c r="L66" s="23" t="str">
         <f>IF(OR(J66="",K66=""),"",J66*K66)</f>
         <v/>
       </c>
@@ -6732,7 +6732,7 @@
       <c r="I67" s="14" t="n"/>
       <c r="J67" s="14" t="n"/>
       <c r="K67" s="23" t="n"/>
-      <c r="L67" s="23">
+      <c r="L67" s="23" t="str">
         <f>IF(OR(J67="",K67=""),"",J67*K67)</f>
         <v/>
       </c>

</xml_diff>